<commit_message>
update: add [29] Aggressive Mode section to input settings guide
Documents all 15 new AggressiveMode inputs introduced in the EA:
AggressiveMode, AggrMinScore, AggrMSSOptional, AggrDispOptional,
AggrDispMinBodyPct, AggrDispMinATRMulti, AggrRequireFVG,
AggrStrictPremDisc, AggrADRMaxPct, AggrStrictKillzone,
AllowContinuation, ExpandKillzones, ScalperMode, ScalperMinScore.
Fixes MergedCell error on ScalperMode row by unmerging before write.

https://claude.ai/code/session_01QqixvfANGqm784CCq6LVR9
</commit_message>
<xml_diff>
--- a/ICT_ATLAS_EA_Input_Guide.xlsx
+++ b/ICT_ATLAS_EA_Input_Guide.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="12">
+  <fonts count="15">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -85,8 +85,23 @@
       <color rgb="00E08030"/>
       <sz val="9"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="8">
+  <fills count="11">
     <fill>
       <patternFill/>
     </fill>
@@ -123,8 +138,23 @@
         <fgColor rgb="0012151F"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001F3864"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F2F2F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFFFF"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="4">
+  <borders count="11">
     <border>
       <left/>
       <right/>
@@ -165,11 +195,85 @@
         <color rgb="003A4070"/>
       </top>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color rgb="003A4070"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="002A3050"/>
+      </right>
+      <top style="medium">
+        <color rgb="003A4070"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color rgb="003A4070"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="003A4070"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="002A3050"/>
+      </right>
+      <top style="medium">
+        <color rgb="003A4070"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="003A4070"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="002A3050"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="002A3050"/>
+      </left>
+      <right style="thin">
+        <color rgb="002A3050"/>
+      </right>
+      <top style="medium">
+        <color rgb="003A4070"/>
+      </top>
+      <bottom/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="002A3050"/>
+      </left>
+      <right style="thin">
+        <color rgb="002A3050"/>
+      </right>
+      <bottom/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -225,6 +329,32 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="10" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="10" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -591,7 +721,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G92"/>
+  <dimension ref="A1:G110"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -609,6 +739,12 @@
           <t>ICT ATLAS EA V1.0  —  Input Settings Guide by Account Size</t>
         </is>
       </c>
+      <c r="B1" s="20" t="n"/>
+      <c r="C1" s="20" t="n"/>
+      <c r="D1" s="20" t="n"/>
+      <c r="E1" s="20" t="n"/>
+      <c r="F1" s="20" t="n"/>
+      <c r="G1" s="21" t="n"/>
     </row>
     <row r="2" ht="22" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
@@ -664,11 +800,12 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="7" t="inlineStr">
+      <c r="A5" s="30" t="inlineStr">
         <is>
           <t xml:space="preserve">  ⚠  XAUUSD minimum viable account: ~$500.  With a 50-pip SL, 0.01 lot = ~$5 risk.  At 1% risk per trade: need $500+.  Accounts below $500 must widen SL limits or use 'Fixed Lot' mode at 0.01.  $50-$100 accounts: use Fixed Lot 0.01 + wider SL tolerance and accept higher % risk per trade.</t>
         </is>
       </c>
+      <c r="G5" s="22" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="3" t="n"/>
@@ -680,11 +817,17 @@
       <c r="G6" s="3" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="8" t="inlineStr">
+      <c r="A7" s="31" t="inlineStr">
         <is>
           <t xml:space="preserve">  SYMBOL PRESET</t>
         </is>
       </c>
+      <c r="B7" s="23" t="n"/>
+      <c r="C7" s="23" t="n"/>
+      <c r="D7" s="23" t="n"/>
+      <c r="E7" s="23" t="n"/>
+      <c r="F7" s="23" t="n"/>
+      <c r="G7" s="24" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="9" t="inlineStr">
@@ -733,11 +876,17 @@
       <c r="G9" s="3" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="8" t="inlineStr">
+      <c r="A10" s="31" t="inlineStr">
         <is>
           <t xml:space="preserve">  [25] RISK MANAGEMENT  ← Most important section</t>
         </is>
       </c>
+      <c r="B10" s="23" t="n"/>
+      <c r="C10" s="23" t="n"/>
+      <c r="D10" s="23" t="n"/>
+      <c r="E10" s="23" t="n"/>
+      <c r="F10" s="23" t="n"/>
+      <c r="G10" s="24" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="9" t="inlineStr">
@@ -971,11 +1120,17 @@
       <c r="G17" s="3" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="8" t="inlineStr">
+      <c r="A18" s="31" t="inlineStr">
         <is>
           <t xml:space="preserve">  [22] ADVANCED TRADE MANAGEMENT  (SL / TP)</t>
         </is>
       </c>
+      <c r="B18" s="23" t="n"/>
+      <c r="C18" s="23" t="n"/>
+      <c r="D18" s="23" t="n"/>
+      <c r="E18" s="23" t="n"/>
+      <c r="F18" s="23" t="n"/>
+      <c r="G18" s="24" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="9" t="inlineStr">
@@ -1468,11 +1623,17 @@
       <c r="G32" s="3" t="n"/>
     </row>
     <row r="33">
-      <c r="A33" s="8" t="inlineStr">
+      <c r="A33" s="31" t="inlineStr">
         <is>
           <t xml:space="preserve">  [24] DAILY LOSS PROTECTION  ← Turn OFF for backtesting</t>
         </is>
       </c>
+      <c r="B33" s="23" t="n"/>
+      <c r="C33" s="23" t="n"/>
+      <c r="D33" s="23" t="n"/>
+      <c r="E33" s="23" t="n"/>
+      <c r="F33" s="23" t="n"/>
+      <c r="G33" s="24" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="9" t="inlineStr">
@@ -1632,11 +1793,17 @@
       <c r="G38" s="3" t="n"/>
     </row>
     <row r="39">
-      <c r="A39" s="8" t="inlineStr">
+      <c r="A39" s="31" t="inlineStr">
         <is>
           <t xml:space="preserve">  [23] DAILY PROFIT LOCK</t>
         </is>
       </c>
+      <c r="B39" s="23" t="n"/>
+      <c r="C39" s="23" t="n"/>
+      <c r="D39" s="23" t="n"/>
+      <c r="E39" s="23" t="n"/>
+      <c r="F39" s="23" t="n"/>
+      <c r="G39" s="24" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="9" t="inlineStr">
@@ -1796,11 +1963,17 @@
       <c r="G44" s="3" t="n"/>
     </row>
     <row r="45">
-      <c r="A45" s="8" t="inlineStr">
+      <c r="A45" s="31" t="inlineStr">
         <is>
           <t xml:space="preserve">  [18] CONFLUENCE SCORING SYSTEM</t>
         </is>
       </c>
+      <c r="B45" s="23" t="n"/>
+      <c r="C45" s="23" t="n"/>
+      <c r="D45" s="23" t="n"/>
+      <c r="E45" s="23" t="n"/>
+      <c r="F45" s="23" t="n"/>
+      <c r="G45" s="24" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="9" t="inlineStr">
@@ -1923,11 +2096,17 @@
       <c r="G49" s="3" t="n"/>
     </row>
     <row r="50">
-      <c r="A50" s="8" t="inlineStr">
+      <c r="A50" s="31" t="inlineStr">
         <is>
           <t xml:space="preserve">  [08] SESSION &amp; KILLZONE ENGINE</t>
         </is>
       </c>
+      <c r="B50" s="23" t="n"/>
+      <c r="C50" s="23" t="n"/>
+      <c r="D50" s="23" t="n"/>
+      <c r="E50" s="23" t="n"/>
+      <c r="F50" s="23" t="n"/>
+      <c r="G50" s="24" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="9" t="inlineStr">
@@ -2161,11 +2340,17 @@
       <c r="G57" s="3" t="n"/>
     </row>
     <row r="58">
-      <c r="A58" s="8" t="inlineStr">
+      <c r="A58" s="31" t="inlineStr">
         <is>
           <t xml:space="preserve">  [13] MARKET CONDITION FILTER</t>
         </is>
       </c>
+      <c r="B58" s="23" t="n"/>
+      <c r="C58" s="23" t="n"/>
+      <c r="D58" s="23" t="n"/>
+      <c r="E58" s="23" t="n"/>
+      <c r="F58" s="23" t="n"/>
+      <c r="G58" s="24" t="n"/>
     </row>
     <row r="59">
       <c r="A59" s="9" t="inlineStr">
@@ -2325,11 +2510,17 @@
       <c r="G63" s="3" t="n"/>
     </row>
     <row r="64">
-      <c r="A64" s="8" t="inlineStr">
+      <c r="A64" s="31" t="inlineStr">
         <is>
           <t xml:space="preserve">  [11] ADR FILTER</t>
         </is>
       </c>
+      <c r="B64" s="23" t="n"/>
+      <c r="C64" s="23" t="n"/>
+      <c r="D64" s="23" t="n"/>
+      <c r="E64" s="23" t="n"/>
+      <c r="F64" s="23" t="n"/>
+      <c r="G64" s="24" t="n"/>
     </row>
     <row r="65">
       <c r="A65" s="9" t="inlineStr">
@@ -2415,11 +2606,17 @@
       <c r="G67" s="3" t="n"/>
     </row>
     <row r="68">
-      <c r="A68" s="8" t="inlineStr">
+      <c r="A68" s="31" t="inlineStr">
         <is>
           <t xml:space="preserve">  [12] NEWS FILTER</t>
         </is>
       </c>
+      <c r="B68" s="23" t="n"/>
+      <c r="C68" s="23" t="n"/>
+      <c r="D68" s="23" t="n"/>
+      <c r="E68" s="23" t="n"/>
+      <c r="F68" s="23" t="n"/>
+      <c r="G68" s="24" t="n"/>
     </row>
     <row r="69">
       <c r="A69" s="9" t="inlineStr">
@@ -2579,11 +2776,17 @@
       <c r="G73" s="3" t="n"/>
     </row>
     <row r="74">
-      <c r="A74" s="8" t="inlineStr">
+      <c r="A74" s="31" t="inlineStr">
         <is>
           <t xml:space="preserve">  TRADE CLOSE RULES</t>
         </is>
       </c>
+      <c r="B74" s="23" t="n"/>
+      <c r="C74" s="23" t="n"/>
+      <c r="D74" s="23" t="n"/>
+      <c r="E74" s="23" t="n"/>
+      <c r="F74" s="23" t="n"/>
+      <c r="G74" s="24" t="n"/>
     </row>
     <row r="75">
       <c r="A75" s="9" t="inlineStr">
@@ -2705,408 +2908,977 @@
       <c r="F78" s="3" t="n"/>
       <c r="G78" s="3" t="n"/>
     </row>
-    <row r="79">
-      <c r="A79" s="8" t="inlineStr">
+    <row r="79" ht="16" customHeight="1">
+      <c r="A79" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  [29] AGGRESSIVE MODE  ← Enables high-frequency ICT trading</t>
+        </is>
+      </c>
+    </row>
+    <row r="80" ht="30" customHeight="1">
+      <c r="A80" s="26" t="inlineStr">
+        <is>
+          <t>AggressiveMode</t>
+        </is>
+      </c>
+      <c r="B80" s="27" t="inlineStr">
+        <is>
+          <t>Master switch for aggressive/high-frequency mode. Relaxes all secondary filters.</t>
+        </is>
+      </c>
+      <c r="C80" s="27" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="D80" s="27" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="E80" s="27" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="F80" s="27" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="G80" s="27" t="inlineStr">
+        <is>
+          <t>Enable for 15-30 trades/day target. Conservative = false</t>
+        </is>
+      </c>
+    </row>
+    <row r="81" ht="30" customHeight="1">
+      <c r="A81" s="28" t="inlineStr">
+        <is>
+          <t>AggrMinScore</t>
+        </is>
+      </c>
+      <c r="B81" s="29" t="inlineStr">
+        <is>
+          <t>Minimum confluence score required when AggressiveMode=true (out of 125).</t>
+        </is>
+      </c>
+      <c r="C81" s="29" t="inlineStr">
+        <is>
+          <t>70</t>
+        </is>
+      </c>
+      <c r="D81" s="29" t="inlineStr">
+        <is>
+          <t>70</t>
+        </is>
+      </c>
+      <c r="E81" s="29" t="inlineStr">
+        <is>
+          <t>70</t>
+        </is>
+      </c>
+      <c r="F81" s="29" t="inlineStr">
+        <is>
+          <t>55</t>
+        </is>
+      </c>
+      <c r="G81" s="29" t="inlineStr">
+        <is>
+          <t>Lower than MinScore — accepts more setups in aggressive mode</t>
+        </is>
+      </c>
+    </row>
+    <row r="82" ht="30" customHeight="1">
+      <c r="A82" s="26" t="inlineStr">
+        <is>
+          <t>AggrMSSOptional</t>
+        </is>
+      </c>
+      <c r="B82" s="27" t="inlineStr">
+        <is>
+          <t>When true, MSS gives half-credit (not required) if sweep + displacement are present.</t>
+        </is>
+      </c>
+      <c r="C82" s="27" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="D82" s="27" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="E82" s="27" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="F82" s="27" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="G82" s="27" t="inlineStr">
+        <is>
+          <t>Removes hard MSS requirement — many valid setups lack textbook MSS</t>
+        </is>
+      </c>
+    </row>
+    <row r="83" ht="30" customHeight="1">
+      <c r="A83" s="28" t="inlineStr">
+        <is>
+          <t>AggrDispOptional</t>
+        </is>
+      </c>
+      <c r="B83" s="29" t="inlineStr">
+        <is>
+          <t>When true, displacement is optional (0 pts, no fail) in aggressive mode.</t>
+        </is>
+      </c>
+      <c r="C83" s="29" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="D83" s="29" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="E83" s="29" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="F83" s="29" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="G83" s="29" t="inlineStr">
+        <is>
+          <t>Keep false — displacement is still a useful quality signal</t>
+        </is>
+      </c>
+    </row>
+    <row r="84" ht="30" customHeight="1">
+      <c r="A84" s="26" t="inlineStr">
+        <is>
+          <t>AggrDispMinBodyPct</t>
+        </is>
+      </c>
+      <c r="B84" s="27" t="inlineStr">
+        <is>
+          <t>Relaxed body % threshold for displacement candles in aggressive mode.</t>
+        </is>
+      </c>
+      <c r="C84" s="27" t="inlineStr">
+        <is>
+          <t>0.60</t>
+        </is>
+      </c>
+      <c r="D84" s="27" t="inlineStr">
+        <is>
+          <t>0.60</t>
+        </is>
+      </c>
+      <c r="E84" s="27" t="inlineStr">
+        <is>
+          <t>0.50</t>
+        </is>
+      </c>
+      <c r="F84" s="27" t="inlineStr">
+        <is>
+          <t>0.40</t>
+        </is>
+      </c>
+      <c r="G84" s="27" t="inlineStr">
+        <is>
+          <t>Conservative default = 0.60. Aggressive = 0.40 (accepts smaller bodies)</t>
+        </is>
+      </c>
+    </row>
+    <row r="85" ht="30" customHeight="1">
+      <c r="A85" s="28" t="inlineStr">
+        <is>
+          <t>AggrDispMinATRMulti</t>
+        </is>
+      </c>
+      <c r="B85" s="29" t="inlineStr">
+        <is>
+          <t>Relaxed ATR multiplier for displacement size in aggressive mode.</t>
+        </is>
+      </c>
+      <c r="C85" s="29" t="inlineStr">
+        <is>
+          <t>1.30</t>
+        </is>
+      </c>
+      <c r="D85" s="29" t="inlineStr">
+        <is>
+          <t>1.30</t>
+        </is>
+      </c>
+      <c r="E85" s="29" t="inlineStr">
+        <is>
+          <t>0.80</t>
+        </is>
+      </c>
+      <c r="F85" s="29" t="inlineStr">
+        <is>
+          <t>0.60</t>
+        </is>
+      </c>
+      <c r="G85" s="29" t="inlineStr">
+        <is>
+          <t>Conservative = 1.3×ATR. Aggressive = 0.6×ATR (accepts smaller moves)</t>
+        </is>
+      </c>
+    </row>
+    <row r="86" ht="30" customHeight="1">
+      <c r="A86" s="26" t="inlineStr">
+        <is>
+          <t>AggrRequireFVG</t>
+        </is>
+      </c>
+      <c r="B86" s="27" t="inlineStr">
+        <is>
+          <t>When false, FVG entry is not required in aggressive mode (market order allowed).</t>
+        </is>
+      </c>
+      <c r="C86" s="27" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="D86" s="27" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="E86" s="27" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="F86" s="27" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="G86" s="27" t="inlineStr">
+        <is>
+          <t>Set false in aggressive — allows entry without waiting for FVG fill</t>
+        </is>
+      </c>
+    </row>
+    <row r="87" ht="30" customHeight="1">
+      <c r="A87" s="28" t="inlineStr">
+        <is>
+          <t>AggrStrictPremDisc</t>
+        </is>
+      </c>
+      <c r="B87" s="29" t="inlineStr">
+        <is>
+          <t>When false, Premium/Discount zone is informational only (no block) in aggressive mode.</t>
+        </is>
+      </c>
+      <c r="C87" s="29" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="D87" s="29" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="E87" s="29" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="F87" s="29" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="G87" s="29" t="inlineStr">
+        <is>
+          <t>Conservative = enforce P/D. Aggressive = treat as scoring only</t>
+        </is>
+      </c>
+    </row>
+    <row r="88" ht="30" customHeight="1">
+      <c r="A88" s="26" t="inlineStr">
+        <is>
+          <t>AggrADRMaxPct</t>
+        </is>
+      </c>
+      <c r="B88" s="27" t="inlineStr">
+        <is>
+          <t>Relaxed ADR completion cap in aggressive mode. Allows entry later in the day.</t>
+        </is>
+      </c>
+      <c r="C88" s="27" t="inlineStr">
+        <is>
+          <t>0.80</t>
+        </is>
+      </c>
+      <c r="D88" s="27" t="inlineStr">
+        <is>
+          <t>0.80</t>
+        </is>
+      </c>
+      <c r="E88" s="27" t="inlineStr">
+        <is>
+          <t>1.00</t>
+        </is>
+      </c>
+      <c r="F88" s="27" t="inlineStr">
+        <is>
+          <t>1.20</t>
+        </is>
+      </c>
+      <c r="G88" s="27" t="inlineStr">
+        <is>
+          <t>120% = entry allowed even if price has moved 120% of ADR already</t>
+        </is>
+      </c>
+    </row>
+    <row r="89" ht="30" customHeight="1">
+      <c r="A89" s="28" t="inlineStr">
+        <is>
+          <t>AggrStrictKillzone</t>
+        </is>
+      </c>
+      <c r="B89" s="29" t="inlineStr">
+        <is>
+          <t>When false, the killzone hard-block is removed in aggressive mode.</t>
+        </is>
+      </c>
+      <c r="C89" s="29" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="D89" s="29" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="E89" s="29" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="F89" s="29" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="G89" s="29" t="inlineStr">
+        <is>
+          <t>Set false to allow entries outside London/NY windows in aggressive mode</t>
+        </is>
+      </c>
+    </row>
+    <row r="90" ht="30" customHeight="1">
+      <c r="A90" s="26" t="inlineStr">
+        <is>
+          <t>AllowContinuation</t>
+        </is>
+      </c>
+      <c r="B90" s="27" t="inlineStr">
+        <is>
+          <t>Allow trades without a sweep when the weekly bias is strongly aligned (half sweep credit).</t>
+        </is>
+      </c>
+      <c r="C90" s="27" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="D90" s="27" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="E90" s="27" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="F90" s="27" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="G90" s="27" t="inlineStr">
+        <is>
+          <t>Continuation trades: bias-aligned moves without a new sweep trigger</t>
+        </is>
+      </c>
+    </row>
+    <row r="91" ht="30" customHeight="1">
+      <c r="A91" s="28" t="inlineStr">
+        <is>
+          <t>ExpandKillzones</t>
+        </is>
+      </c>
+      <c r="B91" s="29" t="inlineStr">
+        <is>
+          <t>Expand all session windows by ±2 hours (e.g. London 07-10 → 05-12 GMT).</t>
+        </is>
+      </c>
+      <c r="C91" s="29" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="D91" s="29" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="E91" s="29" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="F91" s="29" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="G91" s="29" t="inlineStr">
+        <is>
+          <t>More time in-session = more valid entries. Use with aggressive mode</t>
+        </is>
+      </c>
+    </row>
+    <row r="92" ht="30" customHeight="1">
+      <c r="A92" s="26" t="inlineStr">
+        <is>
+          <t>ScalperMode</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>Ultra-aggressive scalper mode. Overrides most filters, uses ScalperMinScore (default 40). Combined with AggressiveMode.</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="G92" t="inlineStr">
+        <is>
+          <t>Experimental. For very high-frequency scalping. All secondary filters bypassed except sweep and score threshold.</t>
+        </is>
+      </c>
+    </row>
+    <row r="93" ht="30" customHeight="1">
+      <c r="A93" s="28" t="inlineStr">
+        <is>
+          <t>ScalperMinScore</t>
+        </is>
+      </c>
+      <c r="B93" s="29" t="inlineStr">
+        <is>
+          <t>Minimum score when ScalperMode=true.</t>
+        </is>
+      </c>
+      <c r="C93" s="29" t="inlineStr">
+        <is>
+          <t>70</t>
+        </is>
+      </c>
+      <c r="D93" s="29" t="inlineStr">
+        <is>
+          <t>70</t>
+        </is>
+      </c>
+      <c r="E93" s="29" t="inlineStr">
+        <is>
+          <t>55</t>
+        </is>
+      </c>
+      <c r="F93" s="29" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="G93" s="29" t="inlineStr">
+        <is>
+          <t>Only active when ScalperMode=true</t>
+        </is>
+      </c>
+    </row>
+    <row r="94" ht="30" customHeight="1">
+      <c r="A94" s="26" t="inlineStr">
+        <is>
+          <t>DebugLogs</t>
+        </is>
+      </c>
+      <c r="B94" s="27" t="inlineStr">
+        <is>
+          <t>Print FVG rejection reasons and setup decisions to the MT5 journal.</t>
+        </is>
+      </c>
+      <c r="C94" s="27" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="D94" s="27" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="E94" s="27" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="F94" s="27" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="G94" s="27" t="inlineStr">
+        <is>
+          <t>Enable when diagnosing why trades are not firing</t>
+        </is>
+      </c>
+    </row>
+    <row r="95" ht="6" customHeight="1"/>
+    <row r="97">
+      <c r="A97" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">  QUICK SUMMARY TABLE</t>
         </is>
       </c>
-    </row>
-    <row r="80">
-      <c r="A80" s="17" t="inlineStr">
+      <c r="B97" s="23" t="n"/>
+      <c r="C97" s="23" t="n"/>
+      <c r="D97" s="23" t="n"/>
+      <c r="E97" s="23" t="n"/>
+      <c r="F97" s="23" t="n"/>
+      <c r="G97" s="24" t="n"/>
+    </row>
+    <row r="98">
+      <c r="A98" s="17" t="inlineStr">
         <is>
           <t>Setting</t>
         </is>
       </c>
-      <c r="B80" s="18" t="inlineStr">
+      <c r="B98" s="18" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
-      <c r="C80" s="19" t="inlineStr">
+      <c r="C98" s="19" t="inlineStr">
         <is>
           <t>$50</t>
         </is>
       </c>
-      <c r="D80" s="19" t="inlineStr">
+      <c r="D98" s="19" t="inlineStr">
         <is>
           <t>$100</t>
         </is>
       </c>
-      <c r="E80" s="19" t="inlineStr">
+      <c r="E98" s="19" t="inlineStr">
         <is>
           <t>$1 000</t>
         </is>
       </c>
-      <c r="F80" s="19" t="inlineStr">
+      <c r="F98" s="19" t="inlineStr">
         <is>
           <t>$10 000</t>
         </is>
       </c>
-      <c r="G80" s="18" t="inlineStr">
+      <c r="G98" s="18" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
     </row>
-    <row r="81">
-      <c r="A81" s="9" t="inlineStr">
+    <row r="99">
+      <c r="A99" s="9" t="inlineStr">
         <is>
           <t>RiskMode</t>
         </is>
       </c>
-      <c r="B81" s="10" t="inlineStr">
+      <c r="B99" s="10" t="inlineStr">
         <is>
           <t>How lot size is calculated</t>
         </is>
       </c>
-      <c r="C81" s="11" t="inlineStr">
+      <c r="C99" s="11" t="inlineStr">
         <is>
           <t>RISK_LOT</t>
         </is>
       </c>
-      <c r="D81" s="11" t="inlineStr">
+      <c r="D99" s="11" t="inlineStr">
         <is>
           <t>RISK_LOT</t>
         </is>
       </c>
-      <c r="E81" s="11" t="inlineStr">
+      <c r="E99" s="11" t="inlineStr">
         <is>
           <t>RISK_PCT</t>
         </is>
       </c>
-      <c r="F81" s="11" t="inlineStr">
+      <c r="F99" s="11" t="inlineStr">
         <is>
           <t>RISK_PCT</t>
         </is>
       </c>
-      <c r="G81" s="12" t="inlineStr"/>
-    </row>
-    <row r="82">
-      <c r="A82" s="13" t="inlineStr">
+      <c r="G99" s="12" t="inlineStr"/>
+    </row>
+    <row r="100">
+      <c r="A100" s="13" t="inlineStr">
         <is>
           <t>RiskPercent / Fixed Lot</t>
         </is>
       </c>
-      <c r="B82" s="14" t="inlineStr">
+      <c r="B100" s="14" t="inlineStr">
         <is>
           <t>Risk per trade</t>
         </is>
       </c>
-      <c r="C82" s="15" t="inlineStr">
+      <c r="C100" s="15" t="inlineStr">
         <is>
           <t>0.01 lot</t>
         </is>
       </c>
-      <c r="D82" s="15" t="inlineStr">
+      <c r="D100" s="15" t="inlineStr">
         <is>
           <t>0.01 lot</t>
         </is>
       </c>
-      <c r="E82" s="15" t="inlineStr">
+      <c r="E100" s="15" t="inlineStr">
         <is>
           <t>1%</t>
         </is>
       </c>
-      <c r="F82" s="15" t="inlineStr">
+      <c r="F100" s="15" t="inlineStr">
         <is>
           <t>0.5%</t>
         </is>
       </c>
-      <c r="G82" s="16" t="inlineStr"/>
-    </row>
-    <row r="83">
-      <c r="A83" s="9" t="inlineStr">
+      <c r="G100" s="16" t="inlineStr"/>
+    </row>
+    <row r="101">
+      <c r="A101" s="9" t="inlineStr">
         <is>
           <t>MaxLotCap</t>
         </is>
       </c>
-      <c r="B83" s="10" t="inlineStr">
+      <c r="B101" s="10" t="inlineStr">
         <is>
           <t>Lot size ceiling</t>
         </is>
       </c>
-      <c r="C83" s="11" t="inlineStr">
+      <c r="C101" s="11" t="inlineStr">
         <is>
           <t>0.01</t>
         </is>
       </c>
-      <c r="D83" s="11" t="inlineStr">
+      <c r="D101" s="11" t="inlineStr">
         <is>
           <t>0.01</t>
         </is>
       </c>
-      <c r="E83" s="11" t="inlineStr">
+      <c r="E101" s="11" t="inlineStr">
         <is>
           <t>0.05</t>
         </is>
       </c>
-      <c r="F83" s="11" t="inlineStr">
+      <c r="F101" s="11" t="inlineStr">
         <is>
           <t>0.50</t>
         </is>
       </c>
-      <c r="G83" s="12" t="inlineStr"/>
-    </row>
-    <row r="84">
-      <c r="A84" s="13" t="inlineStr">
+      <c r="G101" s="12" t="inlineStr"/>
+    </row>
+    <row r="102">
+      <c r="A102" s="13" t="inlineStr">
         <is>
           <t>MaxSLPips</t>
         </is>
       </c>
-      <c r="B84" s="14" t="inlineStr">
+      <c r="B102" s="14" t="inlineStr">
         <is>
           <t>Largest SL allowed</t>
         </is>
       </c>
-      <c r="C84" s="15" t="inlineStr">
+      <c r="C102" s="15" t="inlineStr">
         <is>
           <t>50</t>
         </is>
       </c>
-      <c r="D84" s="15" t="inlineStr">
+      <c r="D102" s="15" t="inlineStr">
         <is>
           <t>50</t>
         </is>
       </c>
-      <c r="E84" s="15" t="inlineStr">
+      <c r="E102" s="15" t="inlineStr">
         <is>
           <t>80</t>
         </is>
       </c>
-      <c r="F84" s="15" t="inlineStr">
+      <c r="F102" s="15" t="inlineStr">
         <is>
           <t>100</t>
         </is>
       </c>
-      <c r="G84" s="16" t="inlineStr"/>
-    </row>
-    <row r="85">
-      <c r="A85" s="9" t="inlineStr">
+      <c r="G102" s="16" t="inlineStr"/>
+    </row>
+    <row r="103">
+      <c r="A103" s="9" t="inlineStr">
         <is>
           <t>MinSLPips</t>
         </is>
       </c>
-      <c r="B85" s="10" t="inlineStr">
+      <c r="B103" s="10" t="inlineStr">
         <is>
           <t>Smallest SL allowed</t>
         </is>
       </c>
-      <c r="C85" s="11" t="inlineStr">
+      <c r="C103" s="11" t="inlineStr">
         <is>
           <t>20</t>
         </is>
       </c>
-      <c r="D85" s="11" t="inlineStr">
+      <c r="D103" s="11" t="inlineStr">
         <is>
           <t>20</t>
         </is>
       </c>
-      <c r="E85" s="11" t="inlineStr">
+      <c r="E103" s="11" t="inlineStr">
         <is>
           <t>15</t>
         </is>
       </c>
-      <c r="F85" s="11" t="inlineStr">
+      <c r="F103" s="11" t="inlineStr">
         <is>
           <t>15</t>
         </is>
       </c>
-      <c r="G85" s="12" t="inlineStr"/>
-    </row>
-    <row r="86">
-      <c r="A86" s="13" t="inlineStr">
+      <c r="G103" s="12" t="inlineStr"/>
+    </row>
+    <row r="104">
+      <c r="A104" s="13" t="inlineStr">
         <is>
           <t>LossProtect_StopR</t>
         </is>
       </c>
-      <c r="B86" s="14" t="inlineStr">
+      <c r="B104" s="14" t="inlineStr">
         <is>
           <t>Daily loss stop (in R)</t>
         </is>
       </c>
-      <c r="C86" s="15" t="inlineStr">
+      <c r="C104" s="15" t="inlineStr">
         <is>
           <t>2R</t>
         </is>
       </c>
-      <c r="D86" s="15" t="inlineStr">
+      <c r="D104" s="15" t="inlineStr">
         <is>
           <t>2R</t>
         </is>
       </c>
-      <c r="E86" s="15" t="inlineStr">
+      <c r="E104" s="15" t="inlineStr">
         <is>
           <t>3R</t>
         </is>
       </c>
-      <c r="F86" s="15" t="inlineStr">
+      <c r="F104" s="15" t="inlineStr">
         <is>
           <t>4R</t>
         </is>
       </c>
-      <c r="G86" s="16" t="inlineStr"/>
-    </row>
-    <row r="87">
-      <c r="A87" s="9" t="inlineStr">
+      <c r="G104" s="16" t="inlineStr"/>
+    </row>
+    <row r="105">
+      <c r="A105" s="9" t="inlineStr">
         <is>
           <t>MaxWeeklyLossR</t>
         </is>
       </c>
-      <c r="B87" s="10" t="inlineStr">
+      <c r="B105" s="10" t="inlineStr">
         <is>
           <t>Weekly loss stop (in R)</t>
         </is>
       </c>
-      <c r="C87" s="11" t="inlineStr">
+      <c r="C105" s="11" t="inlineStr">
         <is>
           <t>3R</t>
         </is>
       </c>
-      <c r="D87" s="11" t="inlineStr">
+      <c r="D105" s="11" t="inlineStr">
         <is>
           <t>3R</t>
         </is>
       </c>
-      <c r="E87" s="11" t="inlineStr">
+      <c r="E105" s="11" t="inlineStr">
         <is>
           <t>6R</t>
         </is>
       </c>
-      <c r="F87" s="11" t="inlineStr">
+      <c r="F105" s="11" t="inlineStr">
         <is>
           <t>8R</t>
         </is>
       </c>
-      <c r="G87" s="12" t="inlineStr"/>
-    </row>
-    <row r="88">
-      <c r="A88" s="13" t="inlineStr">
+      <c r="G105" s="12" t="inlineStr"/>
+    </row>
+    <row r="106">
+      <c r="A106" s="13" t="inlineStr">
         <is>
           <t>MinScore</t>
         </is>
       </c>
-      <c r="B88" s="14" t="inlineStr">
+      <c r="B106" s="14" t="inlineStr">
         <is>
           <t>Confluence gate</t>
         </is>
       </c>
-      <c r="C88" s="15" t="inlineStr">
+      <c r="C106" s="15" t="inlineStr">
         <is>
           <t>70</t>
         </is>
       </c>
-      <c r="D88" s="15" t="inlineStr">
+      <c r="D106" s="15" t="inlineStr">
         <is>
           <t>70</t>
         </is>
       </c>
-      <c r="E88" s="15" t="inlineStr">
+      <c r="E106" s="15" t="inlineStr">
         <is>
           <t>80</t>
         </is>
       </c>
-      <c r="F88" s="15" t="inlineStr">
+      <c r="F106" s="15" t="inlineStr">
         <is>
           <t>85</t>
         </is>
       </c>
-      <c r="G88" s="16" t="inlineStr"/>
-    </row>
-    <row r="89">
-      <c r="A89" s="9" t="inlineStr">
+      <c r="G106" s="16" t="inlineStr"/>
+    </row>
+    <row r="107">
+      <c r="A107" s="9" t="inlineStr">
         <is>
           <t>MaxTradesPerDay</t>
         </is>
       </c>
-      <c r="B89" s="10" t="inlineStr">
+      <c r="B107" s="10" t="inlineStr">
         <is>
           <t>Daily trade limit</t>
         </is>
       </c>
-      <c r="C89" s="11" t="inlineStr">
+      <c r="C107" s="11" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="D89" s="11" t="inlineStr">
+      <c r="D107" s="11" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="E89" s="11" t="inlineStr">
+      <c r="E107" s="11" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="F89" s="11" t="inlineStr">
+      <c r="F107" s="11" t="inlineStr">
         <is>
           <t>5</t>
         </is>
       </c>
-      <c r="G89" s="12" t="inlineStr"/>
-    </row>
-    <row r="90">
-      <c r="A90" s="13" t="inlineStr">
+      <c r="G107" s="12" t="inlineStr"/>
+    </row>
+    <row r="108">
+      <c r="A108" s="13" t="inlineStr">
         <is>
           <t>UseNewsFilter</t>
         </is>
       </c>
-      <c r="B90" s="14" t="inlineStr">
+      <c r="B108" s="14" t="inlineStr">
         <is>
           <t>Block news events</t>
         </is>
       </c>
-      <c r="C90" s="15" t="inlineStr">
-        <is>
-          <t>false</t>
-        </is>
-      </c>
-      <c r="D90" s="15" t="inlineStr">
-        <is>
-          <t>false</t>
-        </is>
-      </c>
-      <c r="E90" s="15" t="inlineStr">
-        <is>
-          <t>false</t>
-        </is>
-      </c>
-      <c r="F90" s="15" t="inlineStr">
-        <is>
-          <t>true</t>
-        </is>
-      </c>
-      <c r="G90" s="16" t="inlineStr"/>
-    </row>
-    <row r="91">
-      <c r="A91" s="3" t="n"/>
-      <c r="B91" s="3" t="n"/>
-      <c r="C91" s="3" t="n"/>
-      <c r="D91" s="3" t="n"/>
-      <c r="E91" s="3" t="n"/>
-      <c r="F91" s="3" t="n"/>
-      <c r="G91" s="3" t="n"/>
-    </row>
-    <row r="92">
-      <c r="A92" s="7" t="inlineStr">
+      <c r="C108" s="15" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="D108" s="15" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="E108" s="15" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="F108" s="15" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="G108" s="16" t="inlineStr"/>
+    </row>
+    <row r="109">
+      <c r="A109" s="3" t="n"/>
+      <c r="B109" s="3" t="n"/>
+      <c r="C109" s="3" t="n"/>
+      <c r="D109" s="3" t="n"/>
+      <c r="E109" s="3" t="n"/>
+      <c r="F109" s="3" t="n"/>
+      <c r="G109" s="3" t="n"/>
+    </row>
+    <row r="110">
+      <c r="A110" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">  ⚠  All other inputs (Bias Engine, Liquidity, MSS, FVG, PDA, P/D, Sessions) can stay at default values for all account sizes. Adjust only when you have 50+ trades of backtest data.</t>
         </is>
       </c>
+      <c r="G110" s="22" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="16">
+  <mergeCells count="15">
     <mergeCell ref="A68:G68"/>
     <mergeCell ref="A58:G58"/>
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="A74:G74"/>
     <mergeCell ref="A18:G18"/>
+    <mergeCell ref="A79:G79"/>
     <mergeCell ref="A45:G45"/>
-    <mergeCell ref="A79:G79"/>
     <mergeCell ref="A39:G39"/>
     <mergeCell ref="A50:G50"/>
-    <mergeCell ref="A92:G92"/>
     <mergeCell ref="A2:G2"/>
     <mergeCell ref="A64:G64"/>
     <mergeCell ref="A7:G7"/>

</xml_diff>

<commit_message>
update: add UseLocalSwingSL, SwingLookback, AggrMaxSLPips, AggrAllowGradeB to input guide
Keeps Excel guide in sync with EA after this session's changes.
Updated both the generator script and regenerated the xlsx.

https://claude.ai/code/session_01QqixvfANGqm784CCq6LVR9
</commit_message>
<xml_diff>
--- a/ICT_ATLAS_EA_Input_Guide.xlsx
+++ b/ICT_ATLAS_EA_Input_Guide.xlsx
@@ -502,7 +502,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G213"/>
+  <dimension ref="A1:G217"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -5366,548 +5366,548 @@
         </is>
       </c>
     </row>
-    <row r="149" ht="16" customHeight="1">
-      <c r="A149" s="8" t="inlineStr">
+    <row r="149" ht="30" customHeight="1">
+      <c r="A149" s="9" t="inlineStr">
+        <is>
+          <t>UseLocalSwingSL</t>
+        </is>
+      </c>
+      <c r="B149" s="9" t="inlineStr">
+        <is>
+          <t>Use local swing high/low for SL instead of PDH/PDL</t>
+        </is>
+      </c>
+      <c r="C149" s="9" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="D149" s="9" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="E149" s="9" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="F149" s="9" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="G149" s="9" t="inlineStr">
+        <is>
+          <t>true = SL placed at nearest swing (5-40 pips). false = SL at PDH/PDL (100-200 pips). Keep true.</t>
+        </is>
+      </c>
+    </row>
+    <row r="150" ht="30" customHeight="1">
+      <c r="A150" s="10" t="inlineStr">
+        <is>
+          <t>SwingLookback</t>
+        </is>
+      </c>
+      <c r="B150" s="10" t="inlineStr">
+        <is>
+          <t>Number of bars back to find local swing high/low for SL</t>
+        </is>
+      </c>
+      <c r="C150" s="10" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="D150" s="10" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="E150" s="10" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="F150" s="10" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="G150" s="10" t="inlineStr">
+        <is>
+          <t>5 bars = ~1.25 hours on M15. Increase to 8-10 for wider SL in volatile markets.</t>
+        </is>
+      </c>
+    </row>
+    <row r="151" ht="16" customHeight="1">
+      <c r="A151" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">  [23] DAILY PROFIT LOCK</t>
         </is>
       </c>
-      <c r="B149" s="8" t="n"/>
-      <c r="C149" s="8" t="n"/>
-      <c r="D149" s="8" t="n"/>
-      <c r="E149" s="8" t="n"/>
-      <c r="F149" s="8" t="n"/>
-      <c r="G149" s="8" t="n"/>
-    </row>
-    <row r="150" ht="30" customHeight="1">
-      <c r="A150" s="9" t="inlineStr">
-        <is>
-          <t>UseProfitLock</t>
-        </is>
-      </c>
-      <c r="B150" s="9" t="inlineStr">
-        <is>
-          <t>Enable automatic profit protection for the day</t>
-        </is>
-      </c>
-      <c r="C150" s="9" t="inlineStr">
-        <is>
-          <t>true</t>
-        </is>
-      </c>
-      <c r="D150" s="9" t="inlineStr">
-        <is>
-          <t>true</t>
-        </is>
-      </c>
-      <c r="E150" s="9" t="inlineStr">
-        <is>
-          <t>true</t>
-        </is>
-      </c>
-      <c r="F150" s="9" t="inlineStr">
-        <is>
-          <t>true</t>
-        </is>
-      </c>
-      <c r="G150" s="9" t="inlineStr">
-        <is>
-          <t>Locks gains after reaching profit target</t>
-        </is>
-      </c>
-    </row>
-    <row r="151" ht="30" customHeight="1">
-      <c r="A151" s="10" t="inlineStr">
-        <is>
-          <t>ProfitLock_ReduceR</t>
-        </is>
-      </c>
-      <c r="B151" s="10" t="inlineStr">
-        <is>
-          <t>Reduce position size after +XR daily profit</t>
-        </is>
-      </c>
-      <c r="C151" s="10" t="inlineStr">
-        <is>
-          <t>3.0</t>
-        </is>
-      </c>
-      <c r="D151" s="10" t="inlineStr">
-        <is>
-          <t>3.0</t>
-        </is>
-      </c>
-      <c r="E151" s="10" t="inlineStr">
-        <is>
-          <t>3.0</t>
-        </is>
-      </c>
-      <c r="F151" s="10" t="inlineStr">
-        <is>
-          <t>3.0</t>
-        </is>
-      </c>
-      <c r="G151" s="10" t="inlineStr">
-        <is>
-          <t>At 3R daily profit, reduce risk by ReducePct%</t>
-        </is>
-      </c>
+      <c r="B151" s="8" t="n"/>
+      <c r="C151" s="8" t="n"/>
+      <c r="D151" s="8" t="n"/>
+      <c r="E151" s="8" t="n"/>
+      <c r="F151" s="8" t="n"/>
+      <c r="G151" s="8" t="n"/>
     </row>
     <row r="152" ht="30" customHeight="1">
       <c r="A152" s="9" t="inlineStr">
         <is>
-          <t>ProfitLock_StopR</t>
+          <t>UseProfitLock</t>
         </is>
       </c>
       <c r="B152" s="9" t="inlineStr">
         <is>
-          <t>Stop trading after +XR daily profit</t>
+          <t>Enable automatic profit protection for the day</t>
         </is>
       </c>
       <c r="C152" s="9" t="inlineStr">
         <is>
-          <t>5.0</t>
+          <t>true</t>
         </is>
       </c>
       <c r="D152" s="9" t="inlineStr">
         <is>
-          <t>5.0</t>
+          <t>true</t>
         </is>
       </c>
       <c r="E152" s="9" t="inlineStr">
         <is>
-          <t>5.0</t>
+          <t>true</t>
         </is>
       </c>
       <c r="F152" s="9" t="inlineStr">
         <is>
-          <t>5.0</t>
+          <t>true</t>
         </is>
       </c>
       <c r="G152" s="9" t="inlineStr">
         <is>
-          <t>At 5R daily profit, no more trades for the day</t>
+          <t>Locks gains after reaching profit target</t>
         </is>
       </c>
     </row>
     <row r="153" ht="30" customHeight="1">
       <c r="A153" s="10" t="inlineStr">
         <is>
+          <t>ProfitLock_ReduceR</t>
+        </is>
+      </c>
+      <c r="B153" s="10" t="inlineStr">
+        <is>
+          <t>Reduce position size after +XR daily profit</t>
+        </is>
+      </c>
+      <c r="C153" s="10" t="inlineStr">
+        <is>
+          <t>3.0</t>
+        </is>
+      </c>
+      <c r="D153" s="10" t="inlineStr">
+        <is>
+          <t>3.0</t>
+        </is>
+      </c>
+      <c r="E153" s="10" t="inlineStr">
+        <is>
+          <t>3.0</t>
+        </is>
+      </c>
+      <c r="F153" s="10" t="inlineStr">
+        <is>
+          <t>3.0</t>
+        </is>
+      </c>
+      <c r="G153" s="10" t="inlineStr">
+        <is>
+          <t>At 3R daily profit, reduce risk by ReducePct%</t>
+        </is>
+      </c>
+    </row>
+    <row r="154" ht="30" customHeight="1">
+      <c r="A154" s="9" t="inlineStr">
+        <is>
+          <t>ProfitLock_StopR</t>
+        </is>
+      </c>
+      <c r="B154" s="9" t="inlineStr">
+        <is>
+          <t>Stop trading after +XR daily profit</t>
+        </is>
+      </c>
+      <c r="C154" s="9" t="inlineStr">
+        <is>
+          <t>5.0</t>
+        </is>
+      </c>
+      <c r="D154" s="9" t="inlineStr">
+        <is>
+          <t>5.0</t>
+        </is>
+      </c>
+      <c r="E154" s="9" t="inlineStr">
+        <is>
+          <t>5.0</t>
+        </is>
+      </c>
+      <c r="F154" s="9" t="inlineStr">
+        <is>
+          <t>5.0</t>
+        </is>
+      </c>
+      <c r="G154" s="9" t="inlineStr">
+        <is>
+          <t>At 5R daily profit, no more trades for the day</t>
+        </is>
+      </c>
+    </row>
+    <row r="155" ht="30" customHeight="1">
+      <c r="A155" s="10" t="inlineStr">
+        <is>
           <t>ProfitLock_ReducePct</t>
         </is>
       </c>
-      <c r="B153" s="10" t="inlineStr">
+      <c r="B155" s="10" t="inlineStr">
         <is>
           <t>Reduce risk by this % when ProfitLock_ReduceR hit</t>
         </is>
       </c>
-      <c r="C153" s="10" t="inlineStr">
+      <c r="C155" s="10" t="inlineStr">
         <is>
           <t>50.0</t>
         </is>
       </c>
-      <c r="D153" s="10" t="inlineStr">
+      <c r="D155" s="10" t="inlineStr">
         <is>
           <t>50.0</t>
         </is>
       </c>
-      <c r="E153" s="10" t="inlineStr">
+      <c r="E155" s="10" t="inlineStr">
         <is>
           <t>50.0</t>
         </is>
       </c>
-      <c r="F153" s="10" t="inlineStr">
+      <c r="F155" s="10" t="inlineStr">
         <is>
           <t>50.0</t>
         </is>
       </c>
-      <c r="G153" s="10" t="inlineStr">
+      <c r="G155" s="10" t="inlineStr">
         <is>
           <t>Trade at 50% of normal risk after hitting reduce level</t>
         </is>
       </c>
     </row>
-    <row r="154" ht="16" customHeight="1">
-      <c r="A154" s="8" t="inlineStr">
+    <row r="156" ht="16" customHeight="1">
+      <c r="A156" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">  [24] DAILY LOSS PROTECTION  ← Turn OFF for backtesting</t>
         </is>
       </c>
-      <c r="B154" s="8" t="n"/>
-      <c r="C154" s="8" t="n"/>
-      <c r="D154" s="8" t="n"/>
-      <c r="E154" s="8" t="n"/>
-      <c r="F154" s="8" t="n"/>
-      <c r="G154" s="8" t="n"/>
-    </row>
-    <row r="155" ht="30" customHeight="1">
-      <c r="A155" s="9" t="inlineStr">
-        <is>
-          <t>UseLossProtect</t>
-        </is>
-      </c>
-      <c r="B155" s="9" t="inlineStr">
-        <is>
-          <t>Enable automatic loss protection for the day</t>
-        </is>
-      </c>
-      <c r="C155" s="9" t="inlineStr">
-        <is>
-          <t>true</t>
-        </is>
-      </c>
-      <c r="D155" s="9" t="inlineStr">
-        <is>
-          <t>true</t>
-        </is>
-      </c>
-      <c r="E155" s="9" t="inlineStr">
-        <is>
-          <t>true</t>
-        </is>
-      </c>
-      <c r="F155" s="9" t="inlineStr">
-        <is>
-          <t>true</t>
-        </is>
-      </c>
-      <c r="G155" s="9" t="inlineStr">
-        <is>
-          <t>Critical for risk control; turn OFF for backtesting</t>
-        </is>
-      </c>
-    </row>
-    <row r="156" ht="30" customHeight="1">
-      <c r="A156" s="10" t="inlineStr">
-        <is>
-          <t>LossProtect_ReduceR</t>
-        </is>
-      </c>
-      <c r="B156" s="10" t="inlineStr">
-        <is>
-          <t>Reduce size after -XR daily loss</t>
-        </is>
-      </c>
-      <c r="C156" s="10" t="inlineStr">
-        <is>
-          <t>2.0</t>
-        </is>
-      </c>
-      <c r="D156" s="10" t="inlineStr">
-        <is>
-          <t>2.0</t>
-        </is>
-      </c>
-      <c r="E156" s="10" t="inlineStr">
-        <is>
-          <t>2.0</t>
-        </is>
-      </c>
-      <c r="F156" s="10" t="inlineStr">
-        <is>
-          <t>2.0</t>
-        </is>
-      </c>
-      <c r="G156" s="10" t="inlineStr">
-        <is>
-          <t>At 2R daily loss, reduce risk by 50%</t>
-        </is>
-      </c>
+      <c r="B156" s="8" t="n"/>
+      <c r="C156" s="8" t="n"/>
+      <c r="D156" s="8" t="n"/>
+      <c r="E156" s="8" t="n"/>
+      <c r="F156" s="8" t="n"/>
+      <c r="G156" s="8" t="n"/>
     </row>
     <row r="157" ht="30" customHeight="1">
       <c r="A157" s="9" t="inlineStr">
         <is>
-          <t>LossProtect_StopR</t>
+          <t>UseLossProtect</t>
         </is>
       </c>
       <c r="B157" s="9" t="inlineStr">
         <is>
-          <t>Stop all trading after -XR daily loss</t>
+          <t>Enable automatic loss protection for the day</t>
         </is>
       </c>
       <c r="C157" s="9" t="inlineStr">
         <is>
-          <t>3.0</t>
+          <t>true</t>
         </is>
       </c>
       <c r="D157" s="9" t="inlineStr">
         <is>
-          <t>3.0</t>
+          <t>true</t>
         </is>
       </c>
       <c r="E157" s="9" t="inlineStr">
         <is>
-          <t>3.0</t>
+          <t>true</t>
         </is>
       </c>
       <c r="F157" s="9" t="inlineStr">
         <is>
-          <t>3.0</t>
+          <t>true</t>
         </is>
       </c>
       <c r="G157" s="9" t="inlineStr">
         <is>
-          <t>At 3R daily loss, no more trades for the day</t>
+          <t>Critical for risk control; turn OFF for backtesting</t>
         </is>
       </c>
     </row>
     <row r="158" ht="30" customHeight="1">
       <c r="A158" s="10" t="inlineStr">
         <is>
+          <t>LossProtect_ReduceR</t>
+        </is>
+      </c>
+      <c r="B158" s="10" t="inlineStr">
+        <is>
+          <t>Reduce size after -XR daily loss</t>
+        </is>
+      </c>
+      <c r="C158" s="10" t="inlineStr">
+        <is>
+          <t>2.0</t>
+        </is>
+      </c>
+      <c r="D158" s="10" t="inlineStr">
+        <is>
+          <t>2.0</t>
+        </is>
+      </c>
+      <c r="E158" s="10" t="inlineStr">
+        <is>
+          <t>2.0</t>
+        </is>
+      </c>
+      <c r="F158" s="10" t="inlineStr">
+        <is>
+          <t>2.0</t>
+        </is>
+      </c>
+      <c r="G158" s="10" t="inlineStr">
+        <is>
+          <t>At 2R daily loss, reduce risk by 50%</t>
+        </is>
+      </c>
+    </row>
+    <row r="159" ht="30" customHeight="1">
+      <c r="A159" s="9" t="inlineStr">
+        <is>
+          <t>LossProtect_StopR</t>
+        </is>
+      </c>
+      <c r="B159" s="9" t="inlineStr">
+        <is>
+          <t>Stop all trading after -XR daily loss</t>
+        </is>
+      </c>
+      <c r="C159" s="9" t="inlineStr">
+        <is>
+          <t>3.0</t>
+        </is>
+      </c>
+      <c r="D159" s="9" t="inlineStr">
+        <is>
+          <t>3.0</t>
+        </is>
+      </c>
+      <c r="E159" s="9" t="inlineStr">
+        <is>
+          <t>3.0</t>
+        </is>
+      </c>
+      <c r="F159" s="9" t="inlineStr">
+        <is>
+          <t>3.0</t>
+        </is>
+      </c>
+      <c r="G159" s="9" t="inlineStr">
+        <is>
+          <t>At 3R daily loss, no more trades for the day</t>
+        </is>
+      </c>
+    </row>
+    <row r="160" ht="30" customHeight="1">
+      <c r="A160" s="10" t="inlineStr">
+        <is>
           <t>MaxWeeklyLossR</t>
         </is>
       </c>
-      <c r="B158" s="10" t="inlineStr">
+      <c r="B160" s="10" t="inlineStr">
         <is>
           <t>Maximum weekly loss in R before stopping</t>
         </is>
       </c>
-      <c r="C158" s="10" t="inlineStr">
+      <c r="C160" s="10" t="inlineStr">
         <is>
           <t>6.0</t>
         </is>
       </c>
-      <c r="D158" s="10" t="inlineStr">
+      <c r="D160" s="10" t="inlineStr">
         <is>
           <t>6.0</t>
         </is>
       </c>
-      <c r="E158" s="10" t="inlineStr">
+      <c r="E160" s="10" t="inlineStr">
         <is>
           <t>6.0</t>
         </is>
       </c>
-      <c r="F158" s="10" t="inlineStr">
+      <c r="F160" s="10" t="inlineStr">
         <is>
           <t>6.0</t>
         </is>
       </c>
-      <c r="G158" s="10" t="inlineStr">
+      <c r="G160" s="10" t="inlineStr">
         <is>
           <t>Weekly circuit breaker; 6R max weekly drawdown</t>
         </is>
       </c>
     </row>
-    <row r="159" ht="16" customHeight="1">
-      <c r="A159" s="8" t="inlineStr">
+    <row r="161" ht="16" customHeight="1">
+      <c r="A161" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">  TRADE CLOSE RULES</t>
         </is>
       </c>
-      <c r="B159" s="8" t="n"/>
-      <c r="C159" s="8" t="n"/>
-      <c r="D159" s="8" t="n"/>
-      <c r="E159" s="8" t="n"/>
-      <c r="F159" s="8" t="n"/>
-      <c r="G159" s="8" t="n"/>
-    </row>
-    <row r="160" ht="30" customHeight="1">
-      <c r="A160" s="9" t="inlineStr">
-        <is>
-          <t>CloseOnFriday</t>
-        </is>
-      </c>
-      <c r="B160" s="9" t="inlineStr">
-        <is>
-          <t>Automatically close all open trades on Friday</t>
-        </is>
-      </c>
-      <c r="C160" s="9" t="inlineStr">
-        <is>
-          <t>true</t>
-        </is>
-      </c>
-      <c r="D160" s="9" t="inlineStr">
-        <is>
-          <t>true</t>
-        </is>
-      </c>
-      <c r="E160" s="9" t="inlineStr">
-        <is>
-          <t>true</t>
-        </is>
-      </c>
-      <c r="F160" s="9" t="inlineStr">
-        <is>
-          <t>true</t>
-        </is>
-      </c>
-      <c r="G160" s="9" t="inlineStr">
-        <is>
-          <t>Avoids weekend gap risk on XAUUSD</t>
-        </is>
-      </c>
-    </row>
-    <row r="161" ht="30" customHeight="1">
-      <c r="A161" s="10" t="inlineStr">
-        <is>
-          <t>FridayCloseHour</t>
-        </is>
-      </c>
-      <c r="B161" s="10" t="inlineStr">
-        <is>
-          <t>GMT hour on Friday to close all trades</t>
-        </is>
-      </c>
-      <c r="C161" s="10" t="inlineStr">
-        <is>
-          <t>14</t>
-        </is>
-      </c>
-      <c r="D161" s="10" t="inlineStr">
-        <is>
-          <t>14</t>
-        </is>
-      </c>
-      <c r="E161" s="10" t="inlineStr">
-        <is>
-          <t>14</t>
-        </is>
-      </c>
-      <c r="F161" s="10" t="inlineStr">
-        <is>
-          <t>14</t>
-        </is>
-      </c>
-      <c r="G161" s="10" t="inlineStr">
-        <is>
-          <t>14:00 GMT = NY open Friday; good liquidity exit</t>
-        </is>
-      </c>
+      <c r="B161" s="8" t="n"/>
+      <c r="C161" s="8" t="n"/>
+      <c r="D161" s="8" t="n"/>
+      <c r="E161" s="8" t="n"/>
+      <c r="F161" s="8" t="n"/>
+      <c r="G161" s="8" t="n"/>
     </row>
     <row r="162" ht="30" customHeight="1">
       <c r="A162" s="9" t="inlineStr">
         <is>
+          <t>CloseOnFriday</t>
+        </is>
+      </c>
+      <c r="B162" s="9" t="inlineStr">
+        <is>
+          <t>Automatically close all open trades on Friday</t>
+        </is>
+      </c>
+      <c r="C162" s="9" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="D162" s="9" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="E162" s="9" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="F162" s="9" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="G162" s="9" t="inlineStr">
+        <is>
+          <t>Avoids weekend gap risk on XAUUSD</t>
+        </is>
+      </c>
+    </row>
+    <row r="163" ht="30" customHeight="1">
+      <c r="A163" s="10" t="inlineStr">
+        <is>
+          <t>FridayCloseHour</t>
+        </is>
+      </c>
+      <c r="B163" s="10" t="inlineStr">
+        <is>
+          <t>GMT hour on Friday to close all trades</t>
+        </is>
+      </c>
+      <c r="C163" s="10" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="D163" s="10" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="E163" s="10" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="F163" s="10" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="G163" s="10" t="inlineStr">
+        <is>
+          <t>14:00 GMT = NY open Friday; good liquidity exit</t>
+        </is>
+      </c>
+    </row>
+    <row r="164" ht="30" customHeight="1">
+      <c r="A164" s="9" t="inlineStr">
+        <is>
           <t>CooldownMinutes</t>
         </is>
       </c>
-      <c r="B162" s="9" t="inlineStr">
+      <c r="B164" s="9" t="inlineStr">
         <is>
           <t>Minimum minutes between two trade entries</t>
         </is>
       </c>
-      <c r="C162" s="9" t="inlineStr">
+      <c r="C164" s="9" t="inlineStr">
         <is>
           <t>30</t>
         </is>
       </c>
-      <c r="D162" s="9" t="inlineStr">
+      <c r="D164" s="9" t="inlineStr">
         <is>
           <t>30</t>
         </is>
       </c>
-      <c r="E162" s="9" t="inlineStr">
+      <c r="E164" s="9" t="inlineStr">
         <is>
           <t>15</t>
         </is>
       </c>
-      <c r="F162" s="9" t="inlineStr">
+      <c r="F164" s="9" t="inlineStr">
         <is>
           <t>15</t>
         </is>
       </c>
-      <c r="G162" s="9" t="inlineStr">
+      <c r="G164" s="9" t="inlineStr">
         <is>
           <t>Prevents over-trading; 15 min in active sessions</t>
         </is>
       </c>
     </row>
-    <row r="163" ht="16" customHeight="1">
-      <c r="A163" s="8" t="inlineStr">
+    <row r="165" ht="16" customHeight="1">
+      <c r="A165" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">  [26] VISUAL CHART TOOLS</t>
         </is>
       </c>
-      <c r="B163" s="8" t="n"/>
-      <c r="C163" s="8" t="n"/>
-      <c r="D163" s="8" t="n"/>
-      <c r="E163" s="8" t="n"/>
-      <c r="F163" s="8" t="n"/>
-      <c r="G163" s="8" t="n"/>
-    </row>
-    <row r="164" ht="30" customHeight="1">
-      <c r="A164" s="10" t="inlineStr">
-        <is>
-          <t>DrawPDH_PDL</t>
-        </is>
-      </c>
-      <c r="B164" s="10" t="inlineStr">
-        <is>
-          <t>Draw Previous Day High and Low lines on chart</t>
-        </is>
-      </c>
-      <c r="C164" s="10" t="inlineStr">
-        <is>
-          <t>true</t>
-        </is>
-      </c>
-      <c r="D164" s="10" t="inlineStr">
-        <is>
-          <t>true</t>
-        </is>
-      </c>
-      <c r="E164" s="10" t="inlineStr">
-        <is>
-          <t>true</t>
-        </is>
-      </c>
-      <c r="F164" s="10" t="inlineStr">
-        <is>
-          <t>true</t>
-        </is>
-      </c>
-      <c r="G164" s="10" t="inlineStr">
-        <is>
-          <t>Key daily reference levels for liquidity</t>
-        </is>
-      </c>
-    </row>
-    <row r="165" ht="30" customHeight="1">
-      <c r="A165" s="9" t="inlineStr">
-        <is>
-          <t>DrawPWH_PWL</t>
-        </is>
-      </c>
-      <c r="B165" s="9" t="inlineStr">
-        <is>
-          <t>Draw Previous Week High and Low lines on chart</t>
-        </is>
-      </c>
-      <c r="C165" s="9" t="inlineStr">
-        <is>
-          <t>true</t>
-        </is>
-      </c>
-      <c r="D165" s="9" t="inlineStr">
-        <is>
-          <t>true</t>
-        </is>
-      </c>
-      <c r="E165" s="9" t="inlineStr">
-        <is>
-          <t>true</t>
-        </is>
-      </c>
-      <c r="F165" s="9" t="inlineStr">
-        <is>
-          <t>true</t>
-        </is>
-      </c>
-      <c r="G165" s="9" t="inlineStr">
-        <is>
-          <t>Weekly reference levels for major sweeps</t>
-        </is>
-      </c>
+      <c r="B165" s="8" t="n"/>
+      <c r="C165" s="8" t="n"/>
+      <c r="D165" s="8" t="n"/>
+      <c r="E165" s="8" t="n"/>
+      <c r="F165" s="8" t="n"/>
+      <c r="G165" s="8" t="n"/>
     </row>
     <row r="166" ht="30" customHeight="1">
       <c r="A166" s="10" t="inlineStr">
         <is>
-          <t>DrawSessionRanges</t>
+          <t>DrawPDH_PDL</t>
         </is>
       </c>
       <c r="B166" s="10" t="inlineStr">
         <is>
-          <t>Draw Asian and London session range boxes</t>
+          <t>Draw Previous Day High and Low lines on chart</t>
         </is>
       </c>
       <c r="C166" s="10" t="inlineStr">
@@ -5932,19 +5932,19 @@
       </c>
       <c r="G166" s="10" t="inlineStr">
         <is>
-          <t>Shows ICT dealing range visually</t>
+          <t>Key daily reference levels for liquidity</t>
         </is>
       </c>
     </row>
     <row r="167" ht="30" customHeight="1">
       <c r="A167" s="9" t="inlineStr">
         <is>
-          <t>DrawFVGZones</t>
+          <t>DrawPWH_PWL</t>
         </is>
       </c>
       <c r="B167" s="9" t="inlineStr">
         <is>
-          <t>Highlight Fair Value Gap zones on chart</t>
+          <t>Draw Previous Week High and Low lines on chart</t>
         </is>
       </c>
       <c r="C167" s="9" t="inlineStr">
@@ -5969,19 +5969,19 @@
       </c>
       <c r="G167" s="9" t="inlineStr">
         <is>
-          <t>Visualizes entry zones</t>
+          <t>Weekly reference levels for major sweeps</t>
         </is>
       </c>
     </row>
     <row r="168" ht="30" customHeight="1">
       <c r="A168" s="10" t="inlineStr">
         <is>
-          <t>DrawOBZones</t>
+          <t>DrawSessionRanges</t>
         </is>
       </c>
       <c r="B168" s="10" t="inlineStr">
         <is>
-          <t>Highlight Order Block zones on chart</t>
+          <t>Draw Asian and London session range boxes</t>
         </is>
       </c>
       <c r="C168" s="10" t="inlineStr">
@@ -6006,19 +6006,19 @@
       </c>
       <c r="G168" s="10" t="inlineStr">
         <is>
-          <t>Visualizes OB entry zones</t>
+          <t>Shows ICT dealing range visually</t>
         </is>
       </c>
     </row>
     <row r="169" ht="30" customHeight="1">
       <c r="A169" s="9" t="inlineStr">
         <is>
-          <t>DrawLiqSweeps</t>
+          <t>DrawFVGZones</t>
         </is>
       </c>
       <c r="B169" s="9" t="inlineStr">
         <is>
-          <t>Mark detected liquidity sweep points</t>
+          <t>Highlight Fair Value Gap zones on chart</t>
         </is>
       </c>
       <c r="C169" s="9" t="inlineStr">
@@ -6043,19 +6043,19 @@
       </c>
       <c r="G169" s="9" t="inlineStr">
         <is>
-          <t>Shows where sweeps occurred</t>
+          <t>Visualizes entry zones</t>
         </is>
       </c>
     </row>
     <row r="170" ht="30" customHeight="1">
       <c r="A170" s="10" t="inlineStr">
         <is>
-          <t>DrawMSSLines</t>
+          <t>DrawOBZones</t>
         </is>
       </c>
       <c r="B170" s="10" t="inlineStr">
         <is>
-          <t>Mark Market Structure Shift levels</t>
+          <t>Highlight Order Block zones on chart</t>
         </is>
       </c>
       <c r="C170" s="10" t="inlineStr">
@@ -6080,19 +6080,19 @@
       </c>
       <c r="G170" s="10" t="inlineStr">
         <is>
-          <t>Shows MSS confirmation levels</t>
+          <t>Visualizes OB entry zones</t>
         </is>
       </c>
     </row>
     <row r="171" ht="30" customHeight="1">
       <c r="A171" s="9" t="inlineStr">
         <is>
-          <t>DrawTargets</t>
+          <t>DrawLiqSweeps</t>
         </is>
       </c>
       <c r="B171" s="9" t="inlineStr">
         <is>
-          <t>Show projected TP1/TP2/TP3 target lines</t>
+          <t>Mark detected liquidity sweep points</t>
         </is>
       </c>
       <c r="C171" s="9" t="inlineStr">
@@ -6117,615 +6117,615 @@
       </c>
       <c r="G171" s="9" t="inlineStr">
         <is>
-          <t>Visualizes reward targets on chart</t>
+          <t>Shows where sweeps occurred</t>
         </is>
       </c>
     </row>
     <row r="172" ht="30" customHeight="1">
       <c r="A172" s="10" t="inlineStr">
         <is>
-          <t>ColorPDH</t>
+          <t>DrawMSSLines</t>
         </is>
       </c>
       <c r="B172" s="10" t="inlineStr">
         <is>
-          <t>Color for Previous Day High line</t>
+          <t>Mark Market Structure Shift levels</t>
         </is>
       </c>
       <c r="C172" s="10" t="inlineStr">
         <is>
-          <t>Lime</t>
+          <t>true</t>
         </is>
       </c>
       <c r="D172" s="10" t="inlineStr">
         <is>
-          <t>Lime</t>
+          <t>true</t>
         </is>
       </c>
       <c r="E172" s="10" t="inlineStr">
         <is>
-          <t>Lime</t>
+          <t>true</t>
         </is>
       </c>
       <c r="F172" s="10" t="inlineStr">
         <is>
-          <t>Lime</t>
+          <t>true</t>
         </is>
       </c>
       <c r="G172" s="10" t="inlineStr">
         <is>
-          <t>Default: Lime green</t>
+          <t>Shows MSS confirmation levels</t>
         </is>
       </c>
     </row>
     <row r="173" ht="30" customHeight="1">
       <c r="A173" s="9" t="inlineStr">
         <is>
-          <t>ColorPDL</t>
+          <t>DrawTargets</t>
         </is>
       </c>
       <c r="B173" s="9" t="inlineStr">
         <is>
-          <t>Color for Previous Day Low line</t>
+          <t>Show projected TP1/TP2/TP3 target lines</t>
         </is>
       </c>
       <c r="C173" s="9" t="inlineStr">
         <is>
-          <t>Tomato</t>
+          <t>true</t>
         </is>
       </c>
       <c r="D173" s="9" t="inlineStr">
         <is>
-          <t>Tomato</t>
+          <t>true</t>
         </is>
       </c>
       <c r="E173" s="9" t="inlineStr">
         <is>
-          <t>Tomato</t>
+          <t>true</t>
         </is>
       </c>
       <c r="F173" s="9" t="inlineStr">
         <is>
-          <t>Tomato</t>
+          <t>true</t>
         </is>
       </c>
       <c r="G173" s="9" t="inlineStr">
         <is>
-          <t>Default: Tomato red</t>
+          <t>Visualizes reward targets on chart</t>
         </is>
       </c>
     </row>
     <row r="174" ht="30" customHeight="1">
       <c r="A174" s="10" t="inlineStr">
         <is>
-          <t>ColorPWH</t>
+          <t>ColorPDH</t>
         </is>
       </c>
       <c r="B174" s="10" t="inlineStr">
         <is>
-          <t>Color for Previous Week High line</t>
+          <t>Color for Previous Day High line</t>
         </is>
       </c>
       <c r="C174" s="10" t="inlineStr">
         <is>
-          <t>Aqua</t>
+          <t>Lime</t>
         </is>
       </c>
       <c r="D174" s="10" t="inlineStr">
         <is>
-          <t>Aqua</t>
+          <t>Lime</t>
         </is>
       </c>
       <c r="E174" s="10" t="inlineStr">
         <is>
-          <t>Aqua</t>
+          <t>Lime</t>
         </is>
       </c>
       <c r="F174" s="10" t="inlineStr">
         <is>
-          <t>Aqua</t>
+          <t>Lime</t>
         </is>
       </c>
       <c r="G174" s="10" t="inlineStr">
         <is>
-          <t>Default: Aqua blue</t>
+          <t>Default: Lime green</t>
         </is>
       </c>
     </row>
     <row r="175" ht="30" customHeight="1">
       <c r="A175" s="9" t="inlineStr">
         <is>
-          <t>ColorPWL</t>
+          <t>ColorPDL</t>
         </is>
       </c>
       <c r="B175" s="9" t="inlineStr">
         <is>
-          <t>Color for Previous Week Low line</t>
+          <t>Color for Previous Day Low line</t>
         </is>
       </c>
       <c r="C175" s="9" t="inlineStr">
         <is>
-          <t>Orange</t>
+          <t>Tomato</t>
         </is>
       </c>
       <c r="D175" s="9" t="inlineStr">
         <is>
-          <t>Orange</t>
+          <t>Tomato</t>
         </is>
       </c>
       <c r="E175" s="9" t="inlineStr">
         <is>
-          <t>Orange</t>
+          <t>Tomato</t>
         </is>
       </c>
       <c r="F175" s="9" t="inlineStr">
         <is>
-          <t>Orange</t>
+          <t>Tomato</t>
         </is>
       </c>
       <c r="G175" s="9" t="inlineStr">
         <is>
-          <t>Default: Orange</t>
+          <t>Default: Tomato red</t>
         </is>
       </c>
     </row>
     <row r="176" ht="30" customHeight="1">
       <c r="A176" s="10" t="inlineStr">
         <is>
-          <t>ColorFVGBull</t>
+          <t>ColorPWH</t>
         </is>
       </c>
       <c r="B176" s="10" t="inlineStr">
         <is>
-          <t>Fill color for Bullish FVG zones</t>
+          <t>Color for Previous Week High line</t>
         </is>
       </c>
       <c r="C176" s="10" t="inlineStr">
         <is>
-          <t>0,80,0</t>
+          <t>Aqua</t>
         </is>
       </c>
       <c r="D176" s="10" t="inlineStr">
         <is>
-          <t>0,80,0</t>
+          <t>Aqua</t>
         </is>
       </c>
       <c r="E176" s="10" t="inlineStr">
         <is>
-          <t>0,80,0</t>
+          <t>Aqua</t>
         </is>
       </c>
       <c r="F176" s="10" t="inlineStr">
         <is>
-          <t>0,80,0</t>
+          <t>Aqua</t>
         </is>
       </c>
       <c r="G176" s="10" t="inlineStr">
         <is>
-          <t>Dark green fill for bullish FVGs</t>
+          <t>Default: Aqua blue</t>
         </is>
       </c>
     </row>
     <row r="177" ht="30" customHeight="1">
       <c r="A177" s="9" t="inlineStr">
         <is>
-          <t>ColorFVGBear</t>
+          <t>ColorPWL</t>
         </is>
       </c>
       <c r="B177" s="9" t="inlineStr">
         <is>
-          <t>Fill color for Bearish FVG zones</t>
+          <t>Color for Previous Week Low line</t>
         </is>
       </c>
       <c r="C177" s="9" t="inlineStr">
         <is>
-          <t>80,0,0</t>
+          <t>Orange</t>
         </is>
       </c>
       <c r="D177" s="9" t="inlineStr">
         <is>
-          <t>80,0,0</t>
+          <t>Orange</t>
         </is>
       </c>
       <c r="E177" s="9" t="inlineStr">
         <is>
-          <t>80,0,0</t>
+          <t>Orange</t>
         </is>
       </c>
       <c r="F177" s="9" t="inlineStr">
         <is>
-          <t>80,0,0</t>
+          <t>Orange</t>
         </is>
       </c>
       <c r="G177" s="9" t="inlineStr">
         <is>
-          <t>Dark red fill for bearish FVGs</t>
+          <t>Default: Orange</t>
         </is>
       </c>
     </row>
     <row r="178" ht="30" customHeight="1">
       <c r="A178" s="10" t="inlineStr">
         <is>
-          <t>ColorOBBull</t>
+          <t>ColorFVGBull</t>
         </is>
       </c>
       <c r="B178" s="10" t="inlineStr">
         <is>
-          <t>Fill color for Bullish Order Block zones</t>
+          <t>Fill color for Bullish FVG zones</t>
         </is>
       </c>
       <c r="C178" s="10" t="inlineStr">
         <is>
-          <t>0,50,100</t>
+          <t>0,80,0</t>
         </is>
       </c>
       <c r="D178" s="10" t="inlineStr">
         <is>
-          <t>0,50,100</t>
+          <t>0,80,0</t>
         </is>
       </c>
       <c r="E178" s="10" t="inlineStr">
         <is>
-          <t>0,50,100</t>
+          <t>0,80,0</t>
         </is>
       </c>
       <c r="F178" s="10" t="inlineStr">
         <is>
-          <t>0,50,100</t>
+          <t>0,80,0</t>
         </is>
       </c>
       <c r="G178" s="10" t="inlineStr">
         <is>
-          <t>Dark blue fill for bullish OBs</t>
+          <t>Dark green fill for bullish FVGs</t>
         </is>
       </c>
     </row>
     <row r="179" ht="30" customHeight="1">
       <c r="A179" s="9" t="inlineStr">
         <is>
+          <t>ColorFVGBear</t>
+        </is>
+      </c>
+      <c r="B179" s="9" t="inlineStr">
+        <is>
+          <t>Fill color for Bearish FVG zones</t>
+        </is>
+      </c>
+      <c r="C179" s="9" t="inlineStr">
+        <is>
+          <t>80,0,0</t>
+        </is>
+      </c>
+      <c r="D179" s="9" t="inlineStr">
+        <is>
+          <t>80,0,0</t>
+        </is>
+      </c>
+      <c r="E179" s="9" t="inlineStr">
+        <is>
+          <t>80,0,0</t>
+        </is>
+      </c>
+      <c r="F179" s="9" t="inlineStr">
+        <is>
+          <t>80,0,0</t>
+        </is>
+      </c>
+      <c r="G179" s="9" t="inlineStr">
+        <is>
+          <t>Dark red fill for bearish FVGs</t>
+        </is>
+      </c>
+    </row>
+    <row r="180" ht="30" customHeight="1">
+      <c r="A180" s="10" t="inlineStr">
+        <is>
+          <t>ColorOBBull</t>
+        </is>
+      </c>
+      <c r="B180" s="10" t="inlineStr">
+        <is>
+          <t>Fill color for Bullish Order Block zones</t>
+        </is>
+      </c>
+      <c r="C180" s="10" t="inlineStr">
+        <is>
+          <t>0,50,100</t>
+        </is>
+      </c>
+      <c r="D180" s="10" t="inlineStr">
+        <is>
+          <t>0,50,100</t>
+        </is>
+      </c>
+      <c r="E180" s="10" t="inlineStr">
+        <is>
+          <t>0,50,100</t>
+        </is>
+      </c>
+      <c r="F180" s="10" t="inlineStr">
+        <is>
+          <t>0,50,100</t>
+        </is>
+      </c>
+      <c r="G180" s="10" t="inlineStr">
+        <is>
+          <t>Dark blue fill for bullish OBs</t>
+        </is>
+      </c>
+    </row>
+    <row r="181" ht="30" customHeight="1">
+      <c r="A181" s="9" t="inlineStr">
+        <is>
           <t>ColorOBBear</t>
         </is>
       </c>
-      <c r="B179" s="9" t="inlineStr">
+      <c r="B181" s="9" t="inlineStr">
         <is>
           <t>Fill color for Bearish Order Block zones</t>
         </is>
       </c>
-      <c r="C179" s="9" t="inlineStr">
+      <c r="C181" s="9" t="inlineStr">
         <is>
           <t>80,30,0</t>
         </is>
       </c>
-      <c r="D179" s="9" t="inlineStr">
+      <c r="D181" s="9" t="inlineStr">
         <is>
           <t>80,30,0</t>
         </is>
       </c>
-      <c r="E179" s="9" t="inlineStr">
+      <c r="E181" s="9" t="inlineStr">
         <is>
           <t>80,30,0</t>
         </is>
       </c>
-      <c r="F179" s="9" t="inlineStr">
+      <c r="F181" s="9" t="inlineStr">
         <is>
           <t>80,30,0</t>
         </is>
       </c>
-      <c r="G179" s="9" t="inlineStr">
+      <c r="G181" s="9" t="inlineStr">
         <is>
           <t>Brown fill for bearish OBs</t>
         </is>
       </c>
     </row>
-    <row r="180" ht="16" customHeight="1">
-      <c r="A180" s="8" t="inlineStr">
+    <row r="182" ht="16" customHeight="1">
+      <c r="A182" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">  [27] DEBUG PANEL</t>
         </is>
       </c>
-      <c r="B180" s="8" t="n"/>
-      <c r="C180" s="8" t="n"/>
-      <c r="D180" s="8" t="n"/>
-      <c r="E180" s="8" t="n"/>
-      <c r="F180" s="8" t="n"/>
-      <c r="G180" s="8" t="n"/>
-    </row>
-    <row r="181" ht="30" customHeight="1">
-      <c r="A181" s="10" t="inlineStr">
-        <is>
-          <t>ShowPanel</t>
-        </is>
-      </c>
-      <c r="B181" s="10" t="inlineStr">
-        <is>
-          <t>Show the ICT ATLAS debug panel on chart</t>
-        </is>
-      </c>
-      <c r="C181" s="10" t="inlineStr">
-        <is>
-          <t>true</t>
-        </is>
-      </c>
-      <c r="D181" s="10" t="inlineStr">
-        <is>
-          <t>true</t>
-        </is>
-      </c>
-      <c r="E181" s="10" t="inlineStr">
-        <is>
-          <t>true</t>
-        </is>
-      </c>
-      <c r="F181" s="10" t="inlineStr">
-        <is>
-          <t>true</t>
-        </is>
-      </c>
-      <c r="G181" s="10" t="inlineStr">
-        <is>
-          <t>Highly recommended — shows real-time EA state</t>
-        </is>
-      </c>
-    </row>
-    <row r="182" ht="30" customHeight="1">
-      <c r="A182" s="9" t="inlineStr">
-        <is>
-          <t>PanelX</t>
-        </is>
-      </c>
-      <c r="B182" s="9" t="inlineStr">
-        <is>
-          <t>Panel horizontal position from left edge (pixels)</t>
-        </is>
-      </c>
-      <c r="C182" s="9" t="inlineStr">
-        <is>
-          <t>12</t>
-        </is>
-      </c>
-      <c r="D182" s="9" t="inlineStr">
-        <is>
-          <t>12</t>
-        </is>
-      </c>
-      <c r="E182" s="9" t="inlineStr">
-        <is>
-          <t>12</t>
-        </is>
-      </c>
-      <c r="F182" s="9" t="inlineStr">
-        <is>
-          <t>12</t>
-        </is>
-      </c>
-      <c r="G182" s="9" t="inlineStr">
-        <is>
-          <t>Adjust if panel overlaps chart elements</t>
-        </is>
-      </c>
+      <c r="B182" s="8" t="n"/>
+      <c r="C182" s="8" t="n"/>
+      <c r="D182" s="8" t="n"/>
+      <c r="E182" s="8" t="n"/>
+      <c r="F182" s="8" t="n"/>
+      <c r="G182" s="8" t="n"/>
     </row>
     <row r="183" ht="30" customHeight="1">
       <c r="A183" s="10" t="inlineStr">
         <is>
-          <t>PanelY</t>
+          <t>ShowPanel</t>
         </is>
       </c>
       <c r="B183" s="10" t="inlineStr">
         <is>
-          <t>Panel vertical position from top edge (pixels)</t>
+          <t>Show the ICT ATLAS debug panel on chart</t>
         </is>
       </c>
       <c r="C183" s="10" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>true</t>
         </is>
       </c>
       <c r="D183" s="10" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>true</t>
         </is>
       </c>
       <c r="E183" s="10" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>true</t>
         </is>
       </c>
       <c r="F183" s="10" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>true</t>
         </is>
       </c>
       <c r="G183" s="10" t="inlineStr">
         <is>
-          <t>Adjust if panel overlaps chart elements</t>
+          <t>Highly recommended — shows real-time EA state</t>
         </is>
       </c>
     </row>
     <row r="184" ht="30" customHeight="1">
       <c r="A184" s="9" t="inlineStr">
         <is>
-          <t>ShowStatPanel</t>
+          <t>PanelX</t>
         </is>
       </c>
       <c r="B184" s="9" t="inlineStr">
         <is>
-          <t>Show statistics section at bottom of panel</t>
+          <t>Panel horizontal position from left edge (pixels)</t>
         </is>
       </c>
       <c r="C184" s="9" t="inlineStr">
         <is>
-          <t>true</t>
+          <t>12</t>
         </is>
       </c>
       <c r="D184" s="9" t="inlineStr">
         <is>
-          <t>true</t>
+          <t>12</t>
         </is>
       </c>
       <c r="E184" s="9" t="inlineStr">
         <is>
-          <t>true</t>
+          <t>12</t>
         </is>
       </c>
       <c r="F184" s="9" t="inlineStr">
         <is>
-          <t>true</t>
+          <t>12</t>
         </is>
       </c>
       <c r="G184" s="9" t="inlineStr">
         <is>
-          <t>Tracks daily P/L, win rate, trade count</t>
+          <t>Adjust if panel overlaps chart elements</t>
         </is>
       </c>
     </row>
     <row r="185" ht="30" customHeight="1">
       <c r="A185" s="10" t="inlineStr">
         <is>
+          <t>PanelY</t>
+        </is>
+      </c>
+      <c r="B185" s="10" t="inlineStr">
+        <is>
+          <t>Panel vertical position from top edge (pixels)</t>
+        </is>
+      </c>
+      <c r="C185" s="10" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="D185" s="10" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="E185" s="10" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="F185" s="10" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="G185" s="10" t="inlineStr">
+        <is>
+          <t>Adjust if panel overlaps chart elements</t>
+        </is>
+      </c>
+    </row>
+    <row r="186" ht="30" customHeight="1">
+      <c r="A186" s="9" t="inlineStr">
+        <is>
+          <t>ShowStatPanel</t>
+        </is>
+      </c>
+      <c r="B186" s="9" t="inlineStr">
+        <is>
+          <t>Show statistics section at bottom of panel</t>
+        </is>
+      </c>
+      <c r="C186" s="9" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="D186" s="9" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="E186" s="9" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="F186" s="9" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="G186" s="9" t="inlineStr">
+        <is>
+          <t>Tracks daily P/L, win rate, trade count</t>
+        </is>
+      </c>
+    </row>
+    <row r="187" ht="30" customHeight="1">
+      <c r="A187" s="10" t="inlineStr">
+        <is>
           <t>DebugLogs</t>
         </is>
       </c>
-      <c r="B185" s="10" t="inlineStr">
+      <c r="B187" s="10" t="inlineStr">
         <is>
           <t>Print detailed FVG and filter decisions to Experts log</t>
         </is>
       </c>
-      <c r="C185" s="10" t="inlineStr">
-        <is>
-          <t>false</t>
-        </is>
-      </c>
-      <c r="D185" s="10" t="inlineStr">
-        <is>
-          <t>false</t>
-        </is>
-      </c>
-      <c r="E185" s="10" t="inlineStr">
-        <is>
-          <t>false</t>
-        </is>
-      </c>
-      <c r="F185" s="10" t="inlineStr">
-        <is>
-          <t>false</t>
-        </is>
-      </c>
-      <c r="G185" s="10" t="inlineStr">
+      <c r="C187" s="10" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="D187" s="10" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="E187" s="10" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="F187" s="10" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="G187" s="10" t="inlineStr">
         <is>
           <t>Enable only when diagnosing why trades are not firing</t>
         </is>
       </c>
     </row>
-    <row r="186" ht="16" customHeight="1">
-      <c r="A186" s="8" t="inlineStr">
+    <row r="188" ht="16" customHeight="1">
+      <c r="A188" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">  [29] AGGRESSIVE MODE  ← Enables high-frequency ICT trading</t>
         </is>
       </c>
-      <c r="B186" s="8" t="n"/>
-      <c r="C186" s="8" t="n"/>
-      <c r="D186" s="8" t="n"/>
-      <c r="E186" s="8" t="n"/>
-      <c r="F186" s="8" t="n"/>
-      <c r="G186" s="8" t="n"/>
-    </row>
-    <row r="187" ht="30" customHeight="1">
-      <c r="A187" s="9" t="inlineStr">
-        <is>
-          <t>AggressiveMode</t>
-        </is>
-      </c>
-      <c r="B187" s="9" t="inlineStr">
-        <is>
-          <t>Master switch for high-frequency / relaxed-filter mode</t>
-        </is>
-      </c>
-      <c r="C187" s="9" t="inlineStr">
-        <is>
-          <t>false</t>
-        </is>
-      </c>
-      <c r="D187" s="9" t="inlineStr">
-        <is>
-          <t>false</t>
-        </is>
-      </c>
-      <c r="E187" s="9" t="inlineStr">
-        <is>
-          <t>false</t>
-        </is>
-      </c>
-      <c r="F187" s="9" t="inlineStr">
-        <is>
-          <t>true</t>
-        </is>
-      </c>
-      <c r="G187" s="9" t="inlineStr">
-        <is>
-          <t>Enable for 15-30 trades/day. Relaxes all secondary filters.</t>
-        </is>
-      </c>
-    </row>
-    <row r="188" ht="30" customHeight="1">
-      <c r="A188" s="10" t="inlineStr">
-        <is>
-          <t>AggrMinScore</t>
-        </is>
-      </c>
-      <c r="B188" s="10" t="inlineStr">
-        <is>
-          <t>Minimum confluence score in aggressive mode</t>
-        </is>
-      </c>
-      <c r="C188" s="10" t="inlineStr">
-        <is>
-          <t>55</t>
-        </is>
-      </c>
-      <c r="D188" s="10" t="inlineStr">
-        <is>
-          <t>55</t>
-        </is>
-      </c>
-      <c r="E188" s="10" t="inlineStr">
-        <is>
-          <t>65</t>
-        </is>
-      </c>
-      <c r="F188" s="10" t="inlineStr">
-        <is>
-          <t>55</t>
-        </is>
-      </c>
-      <c r="G188" s="10" t="inlineStr">
-        <is>
-          <t>Lower than MinScore — accepts more setups in aggressive</t>
-        </is>
-      </c>
+      <c r="B188" s="8" t="n"/>
+      <c r="C188" s="8" t="n"/>
+      <c r="D188" s="8" t="n"/>
+      <c r="E188" s="8" t="n"/>
+      <c r="F188" s="8" t="n"/>
+      <c r="G188" s="8" t="n"/>
     </row>
     <row r="189" ht="30" customHeight="1">
       <c r="A189" s="9" t="inlineStr">
         <is>
-          <t>AggrMSSOptional</t>
+          <t>AggressiveMode</t>
         </is>
       </c>
       <c r="B189" s="9" t="inlineStr">
         <is>
-          <t>MSS gives half-credit (not hard required) in aggressive</t>
+          <t>Master switch for high-frequency / relaxed-filter mode</t>
         </is>
       </c>
       <c r="C189" s="9" t="inlineStr">
         <is>
-          <t>true</t>
+          <t>false</t>
         </is>
       </c>
       <c r="D189" s="9" t="inlineStr">
         <is>
-          <t>true</t>
+          <t>false</t>
         </is>
       </c>
       <c r="E189" s="9" t="inlineStr">
         <is>
-          <t>true</t>
+          <t>false</t>
         </is>
       </c>
       <c r="F189" s="9" t="inlineStr">
@@ -6735,241 +6735,241 @@
       </c>
       <c r="G189" s="9" t="inlineStr">
         <is>
-          <t>Removes hard MSS block; many valid setups lack textbook MSS</t>
+          <t>Enable for 15-30 trades/day. Relaxes all secondary filters.</t>
         </is>
       </c>
     </row>
     <row r="190" ht="30" customHeight="1">
       <c r="A190" s="10" t="inlineStr">
         <is>
-          <t>AggrDispOptional</t>
+          <t>AggrMinScore</t>
         </is>
       </c>
       <c r="B190" s="10" t="inlineStr">
         <is>
-          <t>Displacement is optional (0 pts, no fail) in aggressive</t>
+          <t>Minimum confluence score in aggressive mode</t>
         </is>
       </c>
       <c r="C190" s="10" t="inlineStr">
         <is>
-          <t>false</t>
+          <t>55</t>
         </is>
       </c>
       <c r="D190" s="10" t="inlineStr">
         <is>
-          <t>false</t>
+          <t>55</t>
         </is>
       </c>
       <c r="E190" s="10" t="inlineStr">
         <is>
-          <t>false</t>
+          <t>65</t>
         </is>
       </c>
       <c r="F190" s="10" t="inlineStr">
         <is>
-          <t>false</t>
+          <t>55</t>
         </is>
       </c>
       <c r="G190" s="10" t="inlineStr">
         <is>
-          <t>Keep false — displacement is still a useful quality filter</t>
+          <t>Lower than MinScore — accepts more setups in aggressive</t>
         </is>
       </c>
     </row>
     <row r="191" ht="30" customHeight="1">
       <c r="A191" s="9" t="inlineStr">
         <is>
-          <t>AggrDispMinBodyPct</t>
+          <t>AggrMSSOptional</t>
         </is>
       </c>
       <c r="B191" s="9" t="inlineStr">
         <is>
-          <t>Relaxed body % threshold for displacement in aggressive</t>
+          <t>MSS gives half-credit (not hard required) in aggressive</t>
         </is>
       </c>
       <c r="C191" s="9" t="inlineStr">
         <is>
-          <t>0.40</t>
+          <t>true</t>
         </is>
       </c>
       <c r="D191" s="9" t="inlineStr">
         <is>
-          <t>0.40</t>
+          <t>true</t>
         </is>
       </c>
       <c r="E191" s="9" t="inlineStr">
         <is>
-          <t>0.50</t>
+          <t>true</t>
         </is>
       </c>
       <c r="F191" s="9" t="inlineStr">
         <is>
-          <t>0.40</t>
+          <t>true</t>
         </is>
       </c>
       <c r="G191" s="9" t="inlineStr">
         <is>
-          <t>Conservative = 0.60; Aggressive = 0.40 (accepts more candles)</t>
+          <t>Removes hard MSS block; many valid setups lack textbook MSS</t>
         </is>
       </c>
     </row>
     <row r="192" ht="30" customHeight="1">
       <c r="A192" s="10" t="inlineStr">
         <is>
-          <t>AggrDispMinATRMulti</t>
+          <t>AggrDispOptional</t>
         </is>
       </c>
       <c r="B192" s="10" t="inlineStr">
         <is>
-          <t>Relaxed ATR multiplier for displacement in aggressive</t>
+          <t>Displacement is optional (0 pts, no fail) in aggressive</t>
         </is>
       </c>
       <c r="C192" s="10" t="inlineStr">
         <is>
-          <t>0.60</t>
+          <t>false</t>
         </is>
       </c>
       <c r="D192" s="10" t="inlineStr">
         <is>
-          <t>0.60</t>
+          <t>false</t>
         </is>
       </c>
       <c r="E192" s="10" t="inlineStr">
         <is>
-          <t>0.80</t>
+          <t>false</t>
         </is>
       </c>
       <c r="F192" s="10" t="inlineStr">
         <is>
-          <t>0.60</t>
+          <t>false</t>
         </is>
       </c>
       <c r="G192" s="10" t="inlineStr">
         <is>
-          <t>Conservative = 1.3×ATR; Aggressive = 0.6×ATR</t>
+          <t>Keep false — displacement is still a useful quality filter</t>
         </is>
       </c>
     </row>
     <row r="193" ht="30" customHeight="1">
       <c r="A193" s="9" t="inlineStr">
         <is>
-          <t>AggrRequireFVG</t>
+          <t>AggrDispMinBodyPct</t>
         </is>
       </c>
       <c r="B193" s="9" t="inlineStr">
         <is>
-          <t>Require FVG entry zone in aggressive mode</t>
+          <t>Relaxed body % threshold for displacement in aggressive</t>
         </is>
       </c>
       <c r="C193" s="9" t="inlineStr">
         <is>
-          <t>false</t>
+          <t>0.40</t>
         </is>
       </c>
       <c r="D193" s="9" t="inlineStr">
         <is>
-          <t>false</t>
+          <t>0.40</t>
         </is>
       </c>
       <c r="E193" s="9" t="inlineStr">
         <is>
-          <t>false</t>
+          <t>0.50</t>
         </is>
       </c>
       <c r="F193" s="9" t="inlineStr">
         <is>
-          <t>false</t>
+          <t>0.40</t>
         </is>
       </c>
       <c r="G193" s="9" t="inlineStr">
         <is>
-          <t>Set false in aggressive — allows entry without FVG retrace</t>
+          <t>Conservative = 0.60; Aggressive = 0.40 (accepts more candles)</t>
         </is>
       </c>
     </row>
     <row r="194" ht="30" customHeight="1">
       <c r="A194" s="10" t="inlineStr">
         <is>
-          <t>AggrStrictPremDisc</t>
+          <t>AggrDispMinATRMulti</t>
         </is>
       </c>
       <c r="B194" s="10" t="inlineStr">
         <is>
-          <t>Enforce Premium/Discount zone in aggressive mode</t>
+          <t>Relaxed ATR multiplier for displacement in aggressive</t>
         </is>
       </c>
       <c r="C194" s="10" t="inlineStr">
         <is>
-          <t>false</t>
+          <t>0.60</t>
         </is>
       </c>
       <c r="D194" s="10" t="inlineStr">
         <is>
-          <t>false</t>
+          <t>0.60</t>
         </is>
       </c>
       <c r="E194" s="10" t="inlineStr">
         <is>
-          <t>false</t>
+          <t>0.80</t>
         </is>
       </c>
       <c r="F194" s="10" t="inlineStr">
         <is>
-          <t>false</t>
+          <t>0.60</t>
         </is>
       </c>
       <c r="G194" s="10" t="inlineStr">
         <is>
-          <t>Conservative = enforce P/D; Aggressive = treat as bonus points</t>
+          <t>Conservative = 1.3×ATR; Aggressive = 0.6×ATR</t>
         </is>
       </c>
     </row>
     <row r="195" ht="30" customHeight="1">
       <c r="A195" s="9" t="inlineStr">
         <is>
-          <t>AggrADRMaxPct</t>
+          <t>AggrRequireFVG</t>
         </is>
       </c>
       <c r="B195" s="9" t="inlineStr">
         <is>
-          <t>Relaxed ADR completion cap in aggressive mode</t>
+          <t>Require FVG entry zone in aggressive mode</t>
         </is>
       </c>
       <c r="C195" s="9" t="inlineStr">
         <is>
-          <t>1.20</t>
+          <t>false</t>
         </is>
       </c>
       <c r="D195" s="9" t="inlineStr">
         <is>
-          <t>1.20</t>
+          <t>false</t>
         </is>
       </c>
       <c r="E195" s="9" t="inlineStr">
         <is>
-          <t>1.00</t>
+          <t>false</t>
         </is>
       </c>
       <c r="F195" s="9" t="inlineStr">
         <is>
-          <t>1.20</t>
+          <t>false</t>
         </is>
       </c>
       <c r="G195" s="9" t="inlineStr">
         <is>
-          <t>1.20 = entry allowed even if price moved 120% of normal ADR</t>
+          <t>Set false in aggressive — allows entry without FVG retrace</t>
         </is>
       </c>
     </row>
     <row r="196" ht="30" customHeight="1">
       <c r="A196" s="10" t="inlineStr">
         <is>
-          <t>AggrStrictKillzone</t>
+          <t>AggrStrictPremDisc</t>
         </is>
       </c>
       <c r="B196" s="10" t="inlineStr">
         <is>
-          <t>Require active killzone in aggressive mode</t>
+          <t>Enforce Premium/Discount zone in aggressive mode</t>
         </is>
       </c>
       <c r="C196" s="10" t="inlineStr">
@@ -6994,56 +6994,56 @@
       </c>
       <c r="G196" s="10" t="inlineStr">
         <is>
-          <t>Set false to allow entries outside London/NY windows</t>
+          <t>Conservative = enforce P/D; Aggressive = treat as bonus points</t>
         </is>
       </c>
     </row>
     <row r="197" ht="30" customHeight="1">
       <c r="A197" s="9" t="inlineStr">
         <is>
-          <t>AllowContinuation</t>
+          <t>AggrADRMaxPct</t>
         </is>
       </c>
       <c r="B197" s="9" t="inlineStr">
         <is>
-          <t>Allow trades without a sweep when bias aligned</t>
+          <t>Relaxed ADR completion cap in aggressive mode</t>
         </is>
       </c>
       <c r="C197" s="9" t="inlineStr">
         <is>
-          <t>true</t>
+          <t>1.20</t>
         </is>
       </c>
       <c r="D197" s="9" t="inlineStr">
         <is>
-          <t>true</t>
+          <t>1.20</t>
         </is>
       </c>
       <c r="E197" s="9" t="inlineStr">
         <is>
-          <t>true</t>
+          <t>1.00</t>
         </is>
       </c>
       <c r="F197" s="9" t="inlineStr">
         <is>
-          <t>true</t>
+          <t>1.20</t>
         </is>
       </c>
       <c r="G197" s="9" t="inlineStr">
         <is>
-          <t>Continuation trades: bias-aligned moves without a fresh sweep</t>
+          <t>1.20 = entry allowed even if price moved 120% of normal ADR</t>
         </is>
       </c>
     </row>
     <row r="198" ht="30" customHeight="1">
       <c r="A198" s="10" t="inlineStr">
         <is>
-          <t>ExpandKillzones</t>
+          <t>AggrStrictKillzone</t>
         </is>
       </c>
       <c r="B198" s="10" t="inlineStr">
         <is>
-          <t>Expand all session windows by ±2 hours</t>
+          <t>Require active killzone in aggressive mode</t>
         </is>
       </c>
       <c r="C198" s="10" t="inlineStr">
@@ -7063,301 +7063,317 @@
       </c>
       <c r="F198" s="10" t="inlineStr">
         <is>
-          <t>true</t>
+          <t>false</t>
         </is>
       </c>
       <c r="G198" s="10" t="inlineStr">
         <is>
-          <t>More time in-session = more valid entries in aggressive</t>
+          <t>Set false to allow entries outside London/NY windows</t>
         </is>
       </c>
     </row>
     <row r="199" ht="30" customHeight="1">
       <c r="A199" s="9" t="inlineStr">
         <is>
-          <t>ScalperMode</t>
+          <t>AllowContinuation</t>
         </is>
       </c>
       <c r="B199" s="9" t="inlineStr">
         <is>
-          <t>Ultra-aggressive scalper mode (further relaxed thresholds)</t>
+          <t>Allow trades without a sweep when bias aligned</t>
         </is>
       </c>
       <c r="C199" s="9" t="inlineStr">
         <is>
-          <t>false</t>
+          <t>true</t>
         </is>
       </c>
       <c r="D199" s="9" t="inlineStr">
         <is>
-          <t>false</t>
+          <t>true</t>
         </is>
       </c>
       <c r="E199" s="9" t="inlineStr">
         <is>
-          <t>false</t>
+          <t>true</t>
         </is>
       </c>
       <c r="F199" s="9" t="inlineStr">
         <is>
-          <t>false</t>
+          <t>true</t>
         </is>
       </c>
       <c r="G199" s="9" t="inlineStr">
         <is>
-          <t>Experimental. Uses ScalperMinScore=40; bypasses most filters</t>
+          <t>Continuation trades: bias-aligned moves without a fresh sweep</t>
         </is>
       </c>
     </row>
     <row r="200" ht="30" customHeight="1">
       <c r="A200" s="10" t="inlineStr">
         <is>
+          <t>ExpandKillzones</t>
+        </is>
+      </c>
+      <c r="B200" s="10" t="inlineStr">
+        <is>
+          <t>Expand all session windows by ±2 hours</t>
+        </is>
+      </c>
+      <c r="C200" s="10" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="D200" s="10" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="E200" s="10" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="F200" s="10" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="G200" s="10" t="inlineStr">
+        <is>
+          <t>More time in-session = more valid entries in aggressive</t>
+        </is>
+      </c>
+    </row>
+    <row r="201" ht="30" customHeight="1">
+      <c r="A201" s="9" t="inlineStr">
+        <is>
+          <t>ScalperMode</t>
+        </is>
+      </c>
+      <c r="B201" s="9" t="inlineStr">
+        <is>
+          <t>Ultra-aggressive scalper mode (further relaxed thresholds)</t>
+        </is>
+      </c>
+      <c r="C201" s="9" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="D201" s="9" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="E201" s="9" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="F201" s="9" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="G201" s="9" t="inlineStr">
+        <is>
+          <t>Experimental. Uses ScalperMinScore=40; bypasses most filters</t>
+        </is>
+      </c>
+    </row>
+    <row r="202" ht="30" customHeight="1">
+      <c r="A202" s="10" t="inlineStr">
+        <is>
           <t>ScalperMinScore</t>
         </is>
       </c>
-      <c r="B200" s="10" t="inlineStr">
+      <c r="B202" s="10" t="inlineStr">
         <is>
           <t>Minimum score when ScalperMode=true</t>
         </is>
       </c>
-      <c r="C200" s="10" t="inlineStr">
+      <c r="C202" s="10" t="inlineStr">
         <is>
           <t>40</t>
         </is>
       </c>
-      <c r="D200" s="10" t="inlineStr">
+      <c r="D202" s="10" t="inlineStr">
         <is>
           <t>40</t>
         </is>
       </c>
-      <c r="E200" s="10" t="inlineStr">
+      <c r="E202" s="10" t="inlineStr">
         <is>
           <t>40</t>
         </is>
       </c>
-      <c r="F200" s="10" t="inlineStr">
+      <c r="F202" s="10" t="inlineStr">
         <is>
           <t>40</t>
         </is>
       </c>
-      <c r="G200" s="10" t="inlineStr">
+      <c r="G202" s="10" t="inlineStr">
         <is>
           <t>Only active when ScalperMode=true; very low threshold</t>
         </is>
       </c>
     </row>
-    <row r="201" ht="8" customHeight="1"/>
-    <row r="202" ht="16" customHeight="1">
-      <c r="A202" s="8" t="inlineStr">
+    <row r="203" ht="30" customHeight="1">
+      <c r="A203" s="9" t="inlineStr">
+        <is>
+          <t>AggrMaxSLPips</t>
+        </is>
+      </c>
+      <c r="B203" s="9" t="inlineStr">
+        <is>
+          <t>Maximum allowed SL size in pips when AggressiveMode=true</t>
+        </is>
+      </c>
+      <c r="C203" s="9" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="D203" s="9" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="E203" s="9" t="inlineStr">
+        <is>
+          <t>150</t>
+        </is>
+      </c>
+      <c r="F203" s="9" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="G203" s="9" t="inlineStr">
+        <is>
+          <t>Replaces MaxSLPips cap in aggressive mode. 200 pips allows wide SL from PDH/PDL if UseLocalSwingSL=false.</t>
+        </is>
+      </c>
+    </row>
+    <row r="204" ht="30" customHeight="1">
+      <c r="A204" s="10" t="inlineStr">
+        <is>
+          <t>AggrAllowGradeB</t>
+        </is>
+      </c>
+      <c r="B204" s="10" t="inlineStr">
+        <is>
+          <t>Allow Grade B trades (score 60-79) in aggressive mode</t>
+        </is>
+      </c>
+      <c r="C204" s="10" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="D204" s="10" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="E204" s="10" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="F204" s="10" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="G204" s="10" t="inlineStr">
+        <is>
+          <t>Increases trade frequency. Grade B = valid ICT setup, just fewer confluences than A/A+.</t>
+        </is>
+      </c>
+    </row>
+    <row r="205" ht="8" customHeight="1"/>
+    <row r="206" ht="16" customHeight="1">
+      <c r="A206" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">  QUICK SUMMARY TABLE — Recommended values by account size</t>
         </is>
       </c>
-      <c r="B202" s="8" t="n"/>
-      <c r="C202" s="8" t="n"/>
-      <c r="D202" s="8" t="n"/>
-      <c r="E202" s="8" t="n"/>
-      <c r="F202" s="8" t="n"/>
-      <c r="G202" s="8" t="n"/>
-    </row>
-    <row r="203" ht="18" customHeight="1">
-      <c r="A203" s="5" t="inlineStr">
+      <c r="B206" s="8" t="n"/>
+      <c r="C206" s="8" t="n"/>
+      <c r="D206" s="8" t="n"/>
+      <c r="E206" s="8" t="n"/>
+      <c r="F206" s="8" t="n"/>
+      <c r="G206" s="8" t="n"/>
+    </row>
+    <row r="207" ht="18" customHeight="1">
+      <c r="A207" s="5" t="inlineStr">
         <is>
           <t>Input Name</t>
         </is>
       </c>
-      <c r="B203" s="5" t="inlineStr">
+      <c r="B207" s="5" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
-      <c r="C203" s="5" t="inlineStr">
+      <c r="C207" s="5" t="inlineStr">
         <is>
           <t>$50 acct</t>
         </is>
       </c>
-      <c r="D203" s="5" t="inlineStr">
+      <c r="D207" s="5" t="inlineStr">
         <is>
           <t>$100 acct</t>
         </is>
       </c>
-      <c r="E203" s="5" t="inlineStr">
+      <c r="E207" s="5" t="inlineStr">
         <is>
           <t>$1,000 acct</t>
         </is>
       </c>
-      <c r="F203" s="5" t="inlineStr">
+      <c r="F207" s="5" t="inlineStr">
         <is>
           <t>$10,000 acct</t>
         </is>
       </c>
-      <c r="G203" s="5" t="inlineStr">
+      <c r="G207" s="5" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
-    </row>
-    <row r="204" ht="20" customHeight="1">
-      <c r="A204" s="9" t="inlineStr">
-        <is>
-          <t>RiskMode</t>
-        </is>
-      </c>
-      <c r="B204" s="9" t="inlineStr">
-        <is>
-          <t>Risk calculation method</t>
-        </is>
-      </c>
-      <c r="C204" s="9" t="inlineStr">
-        <is>
-          <t>RISK_LOT</t>
-        </is>
-      </c>
-      <c r="D204" s="9" t="inlineStr">
-        <is>
-          <t>RISK_LOT</t>
-        </is>
-      </c>
-      <c r="E204" s="9" t="inlineStr">
-        <is>
-          <t>RISK_PCT</t>
-        </is>
-      </c>
-      <c r="F204" s="9" t="inlineStr">
-        <is>
-          <t>RISK_PCT</t>
-        </is>
-      </c>
-      <c r="G204" s="9" t="inlineStr"/>
-    </row>
-    <row r="205" ht="20" customHeight="1">
-      <c r="A205" s="10" t="inlineStr">
-        <is>
-          <t>RiskPercent / FixedLot</t>
-        </is>
-      </c>
-      <c r="B205" s="10" t="inlineStr">
-        <is>
-          <t>Risk per trade</t>
-        </is>
-      </c>
-      <c r="C205" s="10" t="inlineStr">
-        <is>
-          <t>0.01 lot</t>
-        </is>
-      </c>
-      <c r="D205" s="10" t="inlineStr">
-        <is>
-          <t>0.01 lot</t>
-        </is>
-      </c>
-      <c r="E205" s="10" t="inlineStr">
-        <is>
-          <t>1.0%</t>
-        </is>
-      </c>
-      <c r="F205" s="10" t="inlineStr">
-        <is>
-          <t>0.5%</t>
-        </is>
-      </c>
-      <c r="G205" s="10" t="inlineStr"/>
-    </row>
-    <row r="206" ht="20" customHeight="1">
-      <c r="A206" s="9" t="inlineStr">
-        <is>
-          <t>MaxLotCap</t>
-        </is>
-      </c>
-      <c r="B206" s="9" t="inlineStr">
-        <is>
-          <t>Lot size ceiling</t>
-        </is>
-      </c>
-      <c r="C206" s="9" t="inlineStr">
-        <is>
-          <t>0.01</t>
-        </is>
-      </c>
-      <c r="D206" s="9" t="inlineStr">
-        <is>
-          <t>0.02</t>
-        </is>
-      </c>
-      <c r="E206" s="9" t="inlineStr">
-        <is>
-          <t>0.10</t>
-        </is>
-      </c>
-      <c r="F206" s="9" t="inlineStr">
-        <is>
-          <t>0.50</t>
-        </is>
-      </c>
-      <c r="G206" s="9" t="inlineStr"/>
-    </row>
-    <row r="207" ht="20" customHeight="1">
-      <c r="A207" s="10" t="inlineStr">
-        <is>
-          <t>MaxSLPips</t>
-        </is>
-      </c>
-      <c r="B207" s="10" t="inlineStr">
-        <is>
-          <t>Maximum stop loss size</t>
-        </is>
-      </c>
-      <c r="C207" s="10" t="inlineStr">
-        <is>
-          <t>80 pips</t>
-        </is>
-      </c>
-      <c r="D207" s="10" t="inlineStr">
-        <is>
-          <t>80 pips</t>
-        </is>
-      </c>
-      <c r="E207" s="10" t="inlineStr">
-        <is>
-          <t>80 pips</t>
-        </is>
-      </c>
-      <c r="F207" s="10" t="inlineStr">
-        <is>
-          <t>80 pips</t>
-        </is>
-      </c>
-      <c r="G207" s="10" t="inlineStr"/>
     </row>
     <row r="208" ht="20" customHeight="1">
       <c r="A208" s="9" t="inlineStr">
         <is>
-          <t>MinSLPips</t>
+          <t>RiskMode</t>
         </is>
       </c>
       <c r="B208" s="9" t="inlineStr">
         <is>
-          <t>Minimum stop loss size</t>
+          <t>Risk calculation method</t>
         </is>
       </c>
       <c r="C208" s="9" t="inlineStr">
         <is>
-          <t>15 pips</t>
+          <t>RISK_LOT</t>
         </is>
       </c>
       <c r="D208" s="9" t="inlineStr">
         <is>
-          <t>15 pips</t>
+          <t>RISK_LOT</t>
         </is>
       </c>
       <c r="E208" s="9" t="inlineStr">
         <is>
-          <t>15 pips</t>
+          <t>RISK_PCT</t>
         </is>
       </c>
       <c r="F208" s="9" t="inlineStr">
         <is>
-          <t>15 pips</t>
+          <t>RISK_PCT</t>
         </is>
       </c>
       <c r="G208" s="9" t="inlineStr"/>
@@ -7365,32 +7381,32 @@
     <row r="209" ht="20" customHeight="1">
       <c r="A209" s="10" t="inlineStr">
         <is>
-          <t>LossProtect_StopR</t>
+          <t>RiskPercent / FixedLot</t>
         </is>
       </c>
       <c r="B209" s="10" t="inlineStr">
         <is>
-          <t>Daily loss limit in R</t>
+          <t>Risk per trade</t>
         </is>
       </c>
       <c r="C209" s="10" t="inlineStr">
         <is>
-          <t>3R</t>
+          <t>0.01 lot</t>
         </is>
       </c>
       <c r="D209" s="10" t="inlineStr">
         <is>
-          <t>3R</t>
+          <t>0.01 lot</t>
         </is>
       </c>
       <c r="E209" s="10" t="inlineStr">
         <is>
-          <t>3R</t>
+          <t>1.0%</t>
         </is>
       </c>
       <c r="F209" s="10" t="inlineStr">
         <is>
-          <t>3R</t>
+          <t>0.5%</t>
         </is>
       </c>
       <c r="G209" s="10" t="inlineStr"/>
@@ -7398,32 +7414,32 @@
     <row r="210" ht="20" customHeight="1">
       <c r="A210" s="9" t="inlineStr">
         <is>
-          <t>MaxWeeklyLossR</t>
+          <t>MaxLotCap</t>
         </is>
       </c>
       <c r="B210" s="9" t="inlineStr">
         <is>
-          <t>Weekly loss limit in R</t>
+          <t>Lot size ceiling</t>
         </is>
       </c>
       <c r="C210" s="9" t="inlineStr">
         <is>
-          <t>6R</t>
+          <t>0.01</t>
         </is>
       </c>
       <c r="D210" s="9" t="inlineStr">
         <is>
-          <t>6R</t>
+          <t>0.02</t>
         </is>
       </c>
       <c r="E210" s="9" t="inlineStr">
         <is>
-          <t>6R</t>
+          <t>0.10</t>
         </is>
       </c>
       <c r="F210" s="9" t="inlineStr">
         <is>
-          <t>6R</t>
+          <t>0.50</t>
         </is>
       </c>
       <c r="G210" s="9" t="inlineStr"/>
@@ -7431,32 +7447,32 @@
     <row r="211" ht="20" customHeight="1">
       <c r="A211" s="10" t="inlineStr">
         <is>
-          <t>MinScore</t>
+          <t>MaxSLPips</t>
         </is>
       </c>
       <c r="B211" s="10" t="inlineStr">
         <is>
-          <t>Minimum confluence score</t>
+          <t>Maximum stop loss size</t>
         </is>
       </c>
       <c r="C211" s="10" t="inlineStr">
         <is>
-          <t>70</t>
+          <t>80 pips</t>
         </is>
       </c>
       <c r="D211" s="10" t="inlineStr">
         <is>
-          <t>70</t>
+          <t>80 pips</t>
         </is>
       </c>
       <c r="E211" s="10" t="inlineStr">
         <is>
-          <t>80</t>
+          <t>80 pips</t>
         </is>
       </c>
       <c r="F211" s="10" t="inlineStr">
         <is>
-          <t>85</t>
+          <t>80 pips</t>
         </is>
       </c>
       <c r="G211" s="10" t="inlineStr"/>
@@ -7464,32 +7480,32 @@
     <row r="212" ht="20" customHeight="1">
       <c r="A212" s="9" t="inlineStr">
         <is>
-          <t>MaxTradesPerDay</t>
+          <t>MinSLPips</t>
         </is>
       </c>
       <c r="B212" s="9" t="inlineStr">
         <is>
-          <t>Max trades per day</t>
+          <t>Minimum stop loss size</t>
         </is>
       </c>
       <c r="C212" s="9" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>15 pips</t>
         </is>
       </c>
       <c r="D212" s="9" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>15 pips</t>
         </is>
       </c>
       <c r="E212" s="9" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>15 pips</t>
         </is>
       </c>
       <c r="F212" s="9" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>15 pips</t>
         </is>
       </c>
       <c r="G212" s="9" t="inlineStr"/>
@@ -7497,52 +7513,186 @@
     <row r="213" ht="20" customHeight="1">
       <c r="A213" s="10" t="inlineStr">
         <is>
+          <t>LossProtect_StopR</t>
+        </is>
+      </c>
+      <c r="B213" s="10" t="inlineStr">
+        <is>
+          <t>Daily loss limit in R</t>
+        </is>
+      </c>
+      <c r="C213" s="10" t="inlineStr">
+        <is>
+          <t>3R</t>
+        </is>
+      </c>
+      <c r="D213" s="10" t="inlineStr">
+        <is>
+          <t>3R</t>
+        </is>
+      </c>
+      <c r="E213" s="10" t="inlineStr">
+        <is>
+          <t>3R</t>
+        </is>
+      </c>
+      <c r="F213" s="10" t="inlineStr">
+        <is>
+          <t>3R</t>
+        </is>
+      </c>
+      <c r="G213" s="10" t="inlineStr"/>
+    </row>
+    <row r="214" ht="20" customHeight="1">
+      <c r="A214" s="9" t="inlineStr">
+        <is>
+          <t>MaxWeeklyLossR</t>
+        </is>
+      </c>
+      <c r="B214" s="9" t="inlineStr">
+        <is>
+          <t>Weekly loss limit in R</t>
+        </is>
+      </c>
+      <c r="C214" s="9" t="inlineStr">
+        <is>
+          <t>6R</t>
+        </is>
+      </c>
+      <c r="D214" s="9" t="inlineStr">
+        <is>
+          <t>6R</t>
+        </is>
+      </c>
+      <c r="E214" s="9" t="inlineStr">
+        <is>
+          <t>6R</t>
+        </is>
+      </c>
+      <c r="F214" s="9" t="inlineStr">
+        <is>
+          <t>6R</t>
+        </is>
+      </c>
+      <c r="G214" s="9" t="inlineStr"/>
+    </row>
+    <row r="215" ht="20" customHeight="1">
+      <c r="A215" s="10" t="inlineStr">
+        <is>
+          <t>MinScore</t>
+        </is>
+      </c>
+      <c r="B215" s="10" t="inlineStr">
+        <is>
+          <t>Minimum confluence score</t>
+        </is>
+      </c>
+      <c r="C215" s="10" t="inlineStr">
+        <is>
+          <t>70</t>
+        </is>
+      </c>
+      <c r="D215" s="10" t="inlineStr">
+        <is>
+          <t>70</t>
+        </is>
+      </c>
+      <c r="E215" s="10" t="inlineStr">
+        <is>
+          <t>80</t>
+        </is>
+      </c>
+      <c r="F215" s="10" t="inlineStr">
+        <is>
+          <t>85</t>
+        </is>
+      </c>
+      <c r="G215" s="10" t="inlineStr"/>
+    </row>
+    <row r="216" ht="20" customHeight="1">
+      <c r="A216" s="9" t="inlineStr">
+        <is>
+          <t>MaxTradesPerDay</t>
+        </is>
+      </c>
+      <c r="B216" s="9" t="inlineStr">
+        <is>
+          <t>Max trades per day</t>
+        </is>
+      </c>
+      <c r="C216" s="9" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="D216" s="9" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="E216" s="9" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="F216" s="9" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="G216" s="9" t="inlineStr"/>
+    </row>
+    <row r="217" ht="20" customHeight="1">
+      <c r="A217" s="10" t="inlineStr">
+        <is>
           <t>AggressiveMode</t>
         </is>
       </c>
-      <c r="B213" s="10" t="inlineStr">
+      <c r="B217" s="10" t="inlineStr">
         <is>
           <t>High-frequency mode</t>
         </is>
       </c>
-      <c r="C213" s="10" t="inlineStr">
-        <is>
-          <t>false</t>
-        </is>
-      </c>
-      <c r="D213" s="10" t="inlineStr">
-        <is>
-          <t>false</t>
-        </is>
-      </c>
-      <c r="E213" s="10" t="inlineStr">
-        <is>
-          <t>false</t>
-        </is>
-      </c>
-      <c r="F213" s="10" t="inlineStr">
+      <c r="C217" s="10" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="D217" s="10" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="E217" s="10" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="F217" s="10" t="inlineStr">
         <is>
           <t>optional</t>
         </is>
       </c>
-      <c r="G213" s="10" t="inlineStr"/>
+      <c r="G217" s="10" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="30">
-    <mergeCell ref="A159:G159"/>
     <mergeCell ref="A135:G135"/>
+    <mergeCell ref="A188:G188"/>
     <mergeCell ref="A106:G106"/>
     <mergeCell ref="A109:G109"/>
+    <mergeCell ref="A206:G206"/>
+    <mergeCell ref="A156:G156"/>
     <mergeCell ref="A72:G72"/>
-    <mergeCell ref="A180:G180"/>
-    <mergeCell ref="A202:G202"/>
+    <mergeCell ref="A165:G165"/>
+    <mergeCell ref="A161:G161"/>
     <mergeCell ref="A9:G9"/>
     <mergeCell ref="A31:G31"/>
     <mergeCell ref="A39:G39"/>
     <mergeCell ref="A83:G83"/>
-    <mergeCell ref="A186:G186"/>
     <mergeCell ref="A15:G15"/>
     <mergeCell ref="A51:G51"/>
+    <mergeCell ref="A182:G182"/>
     <mergeCell ref="A103:G103"/>
     <mergeCell ref="A123:G123"/>
     <mergeCell ref="A1:G1"/>
@@ -7550,14 +7700,12 @@
     <mergeCell ref="A7:G7"/>
     <mergeCell ref="A128:G128"/>
     <mergeCell ref="A75:G75"/>
-    <mergeCell ref="A149:G149"/>
     <mergeCell ref="A56:G56"/>
     <mergeCell ref="A21:G21"/>
-    <mergeCell ref="A154:G154"/>
-    <mergeCell ref="A163:G163"/>
     <mergeCell ref="A26:G26"/>
     <mergeCell ref="A95:G95"/>
     <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A151:G151"/>
     <mergeCell ref="A5:G5"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>